<commit_message>
feat: 100% automation coverage + auto-discovery + VADEMECUM rules
- automation_catalog.json: all 165 automations now have descriptions,
  produces/consumes, LLM details. Zero empties.
- generate_automations_excel.py: auto-discovery for unknown automations
  (Step 1: parse script header, Step 2: claude --print LLM fallback).
  New entries saved to auto_discovered section of catalog.
- VADEMECUM: added point 9 to section 1 (new automation checklist) and
  point 13 to section 11 (LaunchAgent checklist) — both require
  registering in automation_catalog.json.

Coverage: 138/165 from catalog, 27/165 from auto-detection + inline.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/automations-inventory.xlsx
+++ b/docs/automations-inventory.xlsx
@@ -82,12 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-13 23:18 WITA</t>
+          <t>Generated: 2026-04-13 23:50 WITA</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
@@ -1267,7 +1267,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>indexing-daily</t>
+          <t>daily-ops</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1282,12 +1282,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>9:00 WITA</t>
+          <t>8:00 WITA</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Daily indexing sweep for Google Search Console (sequential). Phase 1 - Articles indexing: submit unindexed intel articles to Google Indexing API (max 200/day quota), update apps/evaluator/articles_ind</t>
+          <t>Daily morning operations sweep (sequential). Phase 1 - Business Orchestration: review overnight messages, check CRM pipeline health, identify high-priority clients needing follow-up, flag any urgent p</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>OpenClaw (coder)</t>
+          <t>OpenClaw (main)</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -1330,22 +1330,22 @@
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 01:22</t>
+          <t>2026-04-13 15:29</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>Submitted URLs to Google</t>
+          <t>Telegram daily briefing</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>GSC API, article list</t>
+          <t>CRM, team hours, messages via MCP</t>
         </is>
       </c>
       <c r="R6" s="8" t="inlineStr"/>
@@ -1353,7 +1353,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>nlm-nb1-daily-refresh</t>
+          <t>indexing-daily</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -1368,12 +1368,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>4:30 WITA</t>
+          <t>9:00 WITA</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Run the NLM NB-1 daily refresh pipeline.  1. Execute:    python3 ~/Desktop/nuzantara/scripts/nlm_nb1_daily_refresh.py  2. Report: how many bundles were updated. 3. If failed, send Telegram alert.</t>
+          <t>Daily indexing sweep for Google Search Console (sequential). Phase 1 - Articles indexing: submit unindexed intel articles to Google Indexing API (max 200/day quota), update apps/evaluator/articles_ind</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>OpenClaw (main)</t>
+          <t>OpenClaw (coder)</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
@@ -1406,32 +1406,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 20:30</t>
+          <t>2026-04-13 01:22</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
         </is>
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Updated NB-1 sources</t>
+          <t>Submitted URLs to Google</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Codebase files</t>
+          <t>GSC API, article list</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr"/>
@@ -1439,7 +1439,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>seo-guardian-observe</t>
+          <t>nlm-nb1-daily-refresh</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -1454,12 +1454,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>ogni 40min</t>
+          <t>4:30 WITA</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Run the SEO Guardian observation cycle (Run #25+):  STEP 1 — CHECK SERVICES - Verify backend: curl -s https://nuzantara-rag.fly.dev/health - Verify frontend: curl -I https://balizero.com - Verify llms</t>
+          <t>Run the NLM NB-1 daily refresh pipeline.  1. Execute:    python3 ~/Desktop/nuzantara/scripts/nlm_nb1_daily_refresh.py  2. Report: how many bundles were updated. 3. If failed, send Telegram alert.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1492,32 +1492,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L8" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:01</t>
+          <t>2026-04-12 20:30</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Indexed URLs, coverage metrics</t>
+          <t>Updated NB-1 sources</t>
         </is>
       </c>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>GSC API, coverage_state.json</t>
+          <t>Codebase files</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr"/>
@@ -1525,7 +1525,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>seo-guardian-weekly</t>
+          <t>seo-guardian-observe</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA Lun</t>
+          <t>ogni 40min</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>You are the SEO Guardian weekly LEARN + REPORT phase.  1. exec: cd ~/Desktop/nuzantara &amp;&amp; source apps/backend-rag/venv/bin/activate &amp;&amp; python3 apps/evaluator/seo_guardian_learn.py 2&gt;&amp;1 2. exec: cd ~/D</t>
+          <t>Run the SEO Guardian observation cycle (Run #25+):  STEP 1 — CHECK SERVICES - Verify backend: curl -s https://nuzantara-rag.fly.dev/health - Verify frontend: curl -I https://balizero.com - Verify llms</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1584,26 +1584,26 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 00:00</t>
+          <t>2026-04-13 15:01</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Weekly SEO report, patterns.json</t>
+          <t>Indexed URLs, coverage metrics</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>coverage_state.json, GSC metrics</t>
+          <t>GSC API, coverage_state.json</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr"/>
@@ -1611,7 +1611,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>system-doctor</t>
+          <t>seo-guardian-weekly</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>ogni 4h :0</t>
+          <t>8:00 WITA Lun</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>You are the System Doctor. Diagnose, triage, and fix LOW-risk issues.  Read ~/.openclaw/workspace/autonomous/system-doctor/config.yaml for risk policy.  PHASE 1 — DIAGNOSE (run ALL of these):  1. Back</t>
+          <t>You are the SEO Guardian weekly LEARN + REPORT phase.  1. exec: cd ~/Desktop/nuzantara &amp;&amp; source apps/backend-rag/venv/bin/activate &amp;&amp; python3 apps/evaluator/seo_guardian_learn.py 2&gt;&amp;1 2. exec: cd ~/D</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1670,26 +1670,26 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 12:02</t>
+          <t>2026-04-13 00:00</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>Diagnostic report, auto-fixes</t>
+          <t>Weekly SEO report, patterns.json</t>
         </is>
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Health endpoints, system state</t>
+          <t>coverage_state.json, GSC metrics</t>
         </is>
       </c>
       <c r="R10" s="8" t="inlineStr"/>
@@ -1697,7 +1697,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>t4-monitor-daily</t>
+          <t>system-doctor</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>3:35 WITA</t>
+          <t>ogni 4h :0</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run T4 social media monitor. Execute: bash /Users/nuzantara/Desktop/nuzantara/apps/evaluator/nlm_deep_research/scripts/run_t4_monitor.sh. Check the log at ~/.openclaw/logs/t4_monitor.log for results. </t>
+          <t>You are the System Doctor. Diagnose, triage, and fix LOW-risk issues.  Read ~/.openclaw/workspace/autonomous/system-doctor/config.yaml for risk policy.  PHASE 1 — DIAGNOSE (run ALL of these):  1. Back</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -1750,17 +1750,17 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 19:37</t>
+          <t>2026-04-13 12:02</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
@@ -1770,12 +1770,12 @@
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Social media report</t>
+          <t>Diagnostic report, auto-fixes</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>T4 monitor script output</t>
+          <t>Health endpoints, system state</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr"/>
@@ -1783,7 +1783,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>tech-orchestrator</t>
+          <t>t4-monitor-daily</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>ogni 4h</t>
+          <t>3:35 WITA</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GUARDRAILS (controlla PRIMA di qualsiasi azione):  1. BLACKOUT WINDOW: exec: hour=$(TZ='Asia/Makassar' date +%H); if [ "$hour" -ge 0 ] &amp;&amp; [ "$hour" -lt 3 ]; then echo 'BLACKOUT_00-03_WITA_SKIP'; exit </t>
+          <t xml:space="preserve">Run T4 social media monitor. Execute: bash /Users/nuzantara/Desktop/nuzantara/apps/evaluator/nlm_deep_research/scripts/run_t4_monitor.sh. Check the log at ~/.openclaw/logs/t4_monitor.log for results. </t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1836,17 +1836,17 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L12" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 13:00</t>
+          <t>2026-04-12 19:37</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -1856,12 +1856,12 @@
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Deploy decision, issue list</t>
+          <t>Social media report</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>Git diff, fly status, Core Guardian output</t>
+          <t>T4 monitor script output</t>
         </is>
       </c>
       <c r="R12" s="8" t="inlineStr"/>
@@ -1869,7 +1869,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>weekly-dep-audit</t>
+          <t>tech-orchestrator</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -1884,12 +1884,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>3:30 WITA Lun</t>
+          <t>ogni 4h</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Run weekly dependency audit with auto-patch for safe (patch-only) upgrades.  PHASE 1 — AUDIT: 1. mcporter call nuzantara-mcp-advanced.check_deployment_readiness  2. Python outdated:    exec: source .v</t>
+          <t xml:space="preserve">GUARDRAILS (controlla PRIMA di qualsiasi azione):  1. BLACKOUT WINDOW: exec: hour=$(TZ='Asia/Makassar' date +%H); if [ "$hour" -ge 0 ] &amp;&amp; [ "$hour" -lt 3 ]; then echo 'BLACKOUT_00-03_WITA_SKIP'; exit </t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1928,11 +1928,11 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 19:33</t>
+          <t>2026-04-13 13:00</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Audit report, patched deps</t>
+          <t>Deploy decision, issue list</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>pyproject.toml, pip-audit</t>
+          <t>Git diff, fly status, Core Guardian output</t>
         </is>
       </c>
       <c r="R13" s="8" t="inlineStr"/>
@@ -1955,7 +1955,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>weekly-review</t>
+          <t>weekly-dep-audit</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -1970,12 +1970,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>9:00 WITA Lun</t>
+          <t>3:30 WITA Lun</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Weekly Monday review — business KPIs + technical quality (sequential). Phase 1 - Business Report: summarize week revenue and invoices, new clients onboarded, practice completions, team hours, complian</t>
+          <t>Run weekly dependency audit with auto-patch for safe (patch-only) upgrades.  PHASE 1 — AUDIT: 1. mcporter call nuzantara-mcp-advanced.check_deployment_readiness  2. Python outdated:    exec: source .v</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -2014,26 +2014,26 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 01:39</t>
+          <t>2026-04-12 19:33</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>Telegram weekly report</t>
+          <t>Audit report, patched deps</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>CRM, code quality, Fly.io metrics via MCP</t>
+          <t>pyproject.toml, pip-audit</t>
         </is>
       </c>
       <c r="R14" s="8" t="inlineStr"/>
@@ -2041,7 +2041,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>cell-weekly-report</t>
+          <t>weekly-review</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA Dom</t>
+          <t>9:00 WITA Lun</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — Cell organism weekly report. Task empty.</t>
+          <t>Weekly Monday review — business KPIs + technical quality (sequential). Phase 1 - Business Report: summarize week revenue and invoices, new clients onboarded, practice completions, team hours, complian</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -2086,48 +2086,48 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="L15" s="11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
+          <t>LOCAL</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 00:04</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr"/>
+          <t>2026-04-13 01:39</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+        </is>
+      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Telegram weekly report</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R15" s="8" t="inlineStr">
-        <is>
-          <t>Skipped: empty task.</t>
-        </is>
-      </c>
+          <t>CRM, code quality, Fly.io metrics via MCP</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>daily-ops</t>
+          <t>cell-weekly-report</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2142,12 +2142,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA</t>
+          <t>8:00 WITA Dom</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Daily morning operations sweep (sequential). Phase 1 - Business Orchestration: review overnight messages, check CRM pipeline health, identify high-priority clients needing follow-up, flag any urgent p</t>
+          <t>PLACEHOLDER — Cell organism weekly report. Task empty.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -2172,37 +2172,43 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="L16" s="11" t="inlineStr">
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="L16" s="10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr"/>
+      <c r="M16" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:07</t>
+          <t>2026-04-12 00:04</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr"/>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Telegram daily briefing</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>CRM, team hours, messages via MCP</t>
-        </is>
-      </c>
-      <c r="R16" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>Skipped: empty task.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -2255,12 +2261,12 @@
           <t>LOCAL</t>
         </is>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="L17" s="11" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -2335,17 +2341,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K18" s="10" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M18" s="8" t="inlineStr"/>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 17:10</t>
@@ -2419,17 +2427,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K19" s="10" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M19" s="8" t="inlineStr"/>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:50</t>
@@ -2503,17 +2513,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K20" s="10" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M20" s="8" t="inlineStr"/>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:45</t>
@@ -2587,17 +2599,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K21" s="10" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M21" s="8" t="inlineStr"/>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:20</t>
@@ -2671,17 +2685,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K22" s="10" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L22" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M22" s="8" t="inlineStr"/>
+      <c r="L22" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:35</t>
@@ -2755,17 +2771,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K23" s="10" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M23" s="8" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:30</t>
@@ -2839,17 +2857,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K24" s="10" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M24" s="8" t="inlineStr"/>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:40</t>
@@ -2923,17 +2943,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K25" s="10" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M25" s="8" t="inlineStr"/>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:47</t>
@@ -5577,7 +5599,11 @@
           <t>3:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr"/>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Weekly conversation trainer: trigger conversation-trainer OpenClaw job via cron-runner wrapper. Extracts patterns from recent chats.</t>
+        </is>
+      </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -5616,8 +5642,16 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr"/>
       <c r="O60" s="8" t="inlineStr"/>
-      <c r="P60" s="8" t="inlineStr"/>
-      <c r="Q60" s="8" t="inlineStr"/>
+      <c r="P60" s="8" t="inlineStr">
+        <is>
+          <t>Training patterns</t>
+        </is>
+      </c>
+      <c r="Q60" s="8" t="inlineStr">
+        <is>
+          <t>Recent conversations, OpenClaw gateway</t>
+        </is>
+      </c>
       <c r="R60" s="8" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
@@ -5717,7 +5751,11 @@
           <t>ogni 4min</t>
         </is>
       </c>
-      <c r="E62" s="8" t="inlineStr"/>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>NLM bridge state writer: write heartbeat JSON for Sentinel to monitor NLM bridge daemon.</t>
+        </is>
+      </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -5756,8 +5794,16 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="8" t="inlineStr"/>
       <c r="O62" s="8" t="inlineStr"/>
-      <c r="P62" s="8" t="inlineStr"/>
-      <c r="Q62" s="8" t="inlineStr"/>
+      <c r="P62" s="8" t="inlineStr">
+        <is>
+          <t>State JSON for Sentinel</t>
+        </is>
+      </c>
+      <c r="Q62" s="8" t="inlineStr">
+        <is>
+          <t>System clock</t>
+        </is>
+      </c>
       <c r="R62" s="8" t="inlineStr"/>
     </row>
     <row r="63" ht="30" customHeight="1">
@@ -6237,7 +6283,11 @@
           <t>2:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr"/>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Weekly KG builder: trigger knowledge-graph-builder OpenClaw job via cron-runner wrapper. Ingests entities into Neo4j.</t>
+        </is>
+      </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -6276,8 +6326,16 @@
       <c r="M69" s="8" t="inlineStr"/>
       <c r="N69" s="8" t="inlineStr"/>
       <c r="O69" s="8" t="inlineStr"/>
-      <c r="P69" s="8" t="inlineStr"/>
-      <c r="Q69" s="8" t="inlineStr"/>
+      <c r="P69" s="8" t="inlineStr">
+        <is>
+          <t>KG entities (Neo4j)</t>
+        </is>
+      </c>
+      <c r="Q69" s="8" t="inlineStr">
+        <is>
+          <t>Conversation data, OpenClaw gateway</t>
+        </is>
+      </c>
       <c r="R69" s="8" t="inlineStr"/>
     </row>
     <row r="70" ht="30" customHeight="1">
@@ -6453,7 +6511,11 @@
           <t>3:30 WITA giorno 1,15</t>
         </is>
       </c>
-      <c r="E72" s="8" t="inlineStr"/>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>Cache cleanup: npm + pip + brew cache purge. Runs 1st and 15th of each month.</t>
+        </is>
+      </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -6492,8 +6554,16 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="8" t="inlineStr"/>
       <c r="O72" s="8" t="inlineStr"/>
-      <c r="P72" s="8" t="inlineStr"/>
-      <c r="Q72" s="8" t="inlineStr"/>
+      <c r="P72" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q72" s="8" t="inlineStr">
+        <is>
+          <t>npm/pip/brew caches</t>
+        </is>
+      </c>
       <c r="R72" s="8" t="inlineStr"/>
     </row>
     <row r="73" ht="30" customHeight="1">
@@ -8949,7 +9019,11 @@
           <t>ogni ora :0</t>
         </is>
       </c>
-      <c r="E105" s="8" t="inlineStr"/>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>Pro heartbeat: write timestamp locally + push to Air via SSH. Hourly dead-man switch.</t>
+        </is>
+      </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -8988,8 +9062,16 @@
       <c r="M105" s="8" t="inlineStr"/>
       <c r="N105" s="8" t="inlineStr"/>
       <c r="O105" s="8" t="inlineStr"/>
-      <c r="P105" s="8" t="inlineStr"/>
-      <c r="Q105" s="8" t="inlineStr"/>
+      <c r="P105" s="8" t="inlineStr">
+        <is>
+          <t>Heartbeat file on both nodes</t>
+        </is>
+      </c>
+      <c r="Q105" s="8" t="inlineStr">
+        <is>
+          <t>SSH to Air</t>
+        </is>
+      </c>
       <c r="R105" s="8" t="inlineStr"/>
     </row>
     <row r="106" ht="30" customHeight="1">
@@ -9257,16 +9339,16 @@
         </is>
       </c>
       <c r="M2" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:29</t>
+          <t>2026-04-13 15:35</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>Error: All models failed (2): ollama/qwen3:4b: LLM request timed out. (unknown) | google-gemini-cli/</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
@@ -9343,11 +9425,11 @@
         </is>
       </c>
       <c r="M3" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 14:54</t>
+          <t>2026-04-13 15:24</t>
         </is>
       </c>
       <c r="O3" s="8" t="inlineStr">
@@ -9515,16 +9597,16 @@
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:42</t>
+          <t>2026-04-13 15:46</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>cron: job execution timed out</t>
         </is>
       </c>
       <c r="P5" s="8" t="inlineStr">
@@ -9930,7 +10012,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -10010,7 +10092,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K11" s="11" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -10090,7 +10172,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -10170,7 +10252,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K13" s="11" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -11524,7 +11606,11 @@
           <t>3:30 WITA giorno 1,15</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr"/>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Orphan crontab entry — incomplete script reference. Likely a broken entry.</t>
+        </is>
+      </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11565,7 +11651,11 @@
       <c r="O32" s="8" t="inlineStr"/>
       <c r="P32" s="8" t="inlineStr"/>
       <c r="Q32" s="8" t="inlineStr"/>
-      <c r="R32" s="8" t="inlineStr"/>
+      <c r="R32" s="8" t="inlineStr">
+        <is>
+          <t>AUDIT: remove or fix in crontab</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
@@ -11588,7 +11678,11 @@
           <t>7:30 WITA</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr"/>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Auto practice creator: POST to Fly.io API to auto-create practices for expiring visas at T-60 days.</t>
+        </is>
+      </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11627,8 +11721,16 @@
       <c r="M33" s="8" t="inlineStr"/>
       <c r="N33" s="8" t="inlineStr"/>
       <c r="O33" s="8" t="inlineStr"/>
-      <c r="P33" s="8" t="inlineStr"/>
-      <c r="Q33" s="8" t="inlineStr"/>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>New CRM practices</t>
+        </is>
+      </c>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R33" s="8" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
@@ -11652,7 +11754,11 @@
           <t>0:00 WITA</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr"/>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>All notifiers: trigger visa expiry, unpaid invoices, stale practice alerts via backend API.</t>
+        </is>
+      </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11691,8 +11797,16 @@
       <c r="M34" s="8" t="inlineStr"/>
       <c r="N34" s="8" t="inlineStr"/>
       <c r="O34" s="8" t="inlineStr"/>
-      <c r="P34" s="8" t="inlineStr"/>
-      <c r="Q34" s="8" t="inlineStr"/>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>Client alerts (WhatsApp/email/Telegram)</t>
+        </is>
+      </c>
+      <c r="Q34" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R34" s="8" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
@@ -11716,7 +11830,11 @@
           <t>0:05 WITA</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr"/>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Birthday notifier: send birthday greetings to clients via backend API.</t>
+        </is>
+      </c>
       <c r="F35" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11755,8 +11873,16 @@
       <c r="M35" s="8" t="inlineStr"/>
       <c r="N35" s="8" t="inlineStr"/>
       <c r="O35" s="8" t="inlineStr"/>
-      <c r="P35" s="8" t="inlineStr"/>
-      <c r="Q35" s="8" t="inlineStr"/>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>Birthday greeting messages</t>
+        </is>
+      </c>
+      <c r="Q35" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R35" s="8" t="inlineStr"/>
     </row>
     <row r="36" ht="30" customHeight="1">
@@ -11780,7 +11906,11 @@
           <t>ogni 15min</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr"/>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Welcome pending: send welcome emails to new clients after 30min delay. Every 15min.</t>
+        </is>
+      </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11819,8 +11949,16 @@
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="8" t="inlineStr"/>
       <c r="O36" s="8" t="inlineStr"/>
-      <c r="P36" s="8" t="inlineStr"/>
-      <c r="Q36" s="8" t="inlineStr"/>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>Welcome emails</t>
+        </is>
+      </c>
+      <c r="Q36" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R36" s="8" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
@@ -11844,7 +11982,11 @@
           <t>2:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr"/>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Weekly audit trail cleanup: prune old audit log entries on Air.</t>
+        </is>
+      </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -11883,8 +12025,16 @@
       <c r="M37" s="8" t="inlineStr"/>
       <c r="N37" s="8" t="inlineStr"/>
       <c r="O37" s="8" t="inlineStr"/>
-      <c r="P37" s="8" t="inlineStr"/>
-      <c r="Q37" s="8" t="inlineStr"/>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q37" s="8" t="inlineStr">
+        <is>
+          <t>Audit log files</t>
+        </is>
+      </c>
       <c r="R37" s="8" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
@@ -12212,7 +12362,11 @@
           <t>4:00 WITA</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr"/>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>MOS daily backup: copy memory.db to timestamped backup file.</t>
+        </is>
+      </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12251,8 +12405,16 @@
       <c r="M42" s="8" t="inlineStr"/>
       <c r="N42" s="8" t="inlineStr"/>
       <c r="O42" s="8" t="inlineStr"/>
-      <c r="P42" s="8" t="inlineStr"/>
-      <c r="Q42" s="8" t="inlineStr"/>
+      <c r="P42" s="8" t="inlineStr">
+        <is>
+          <t>Memory DB backup</t>
+        </is>
+      </c>
+      <c r="Q42" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/memory.db</t>
+        </is>
+      </c>
       <c r="R42" s="8" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
@@ -12276,7 +12438,11 @@
           <t>23:00 WITA</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr"/>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>CRM automation engine: quality checks, document follow-up, renewal processing. Runs nightly on Air.</t>
+        </is>
+      </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12315,8 +12481,16 @@
       <c r="M43" s="8" t="inlineStr"/>
       <c r="N43" s="8" t="inlineStr"/>
       <c r="O43" s="8" t="inlineStr"/>
-      <c r="P43" s="8" t="inlineStr"/>
-      <c r="Q43" s="8" t="inlineStr"/>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>CRM updates, follow-up tasks</t>
+        </is>
+      </c>
+      <c r="Q43" s="8" t="inlineStr">
+        <is>
+          <t>Backend API CRM data</t>
+        </is>
+      </c>
       <c r="R43" s="8" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
@@ -12340,7 +12514,11 @@
           <t>23:00 WITA</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr"/>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Cron wrapper: universal wrapper that adds logging, locking, timeout, and Telegram alerts to any cron script.</t>
+        </is>
+      </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12379,8 +12557,16 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="8" t="inlineStr"/>
       <c r="O44" s="8" t="inlineStr"/>
-      <c r="P44" s="8" t="inlineStr"/>
-      <c r="Q44" s="8" t="inlineStr"/>
+      <c r="P44" s="8" t="inlineStr">
+        <is>
+          <t>Structured logs, state files</t>
+        </is>
+      </c>
+      <c r="Q44" s="8" t="inlineStr">
+        <is>
+          <t>Wrapped script output</t>
+        </is>
+      </c>
       <c r="R44" s="8" t="inlineStr"/>
     </row>
     <row r="45" ht="30" customHeight="1">
@@ -12480,7 +12666,11 @@
           <t>5:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr"/>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>MOS backup pruning: delete memory backups older than 30 days.</t>
+        </is>
+      </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12519,8 +12709,16 @@
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="8" t="inlineStr"/>
       <c r="O46" s="8" t="inlineStr"/>
-      <c r="P46" s="8" t="inlineStr"/>
-      <c r="Q46" s="8" t="inlineStr"/>
+      <c r="P46" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q46" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/backups/</t>
+        </is>
+      </c>
       <c r="R46" s="8" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
@@ -12544,7 +12742,11 @@
           <t>3:20 WITA</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr"/>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Fly PG backup (Air): pg_dump from Fly.io PG tunnel to local backup. Separate from Pro fly-backup.sh.</t>
+        </is>
+      </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12583,8 +12785,16 @@
       <c r="M47" s="8" t="inlineStr"/>
       <c r="N47" s="8" t="inlineStr"/>
       <c r="O47" s="8" t="inlineStr"/>
-      <c r="P47" s="8" t="inlineStr"/>
-      <c r="Q47" s="8" t="inlineStr"/>
+      <c r="P47" s="8" t="inlineStr">
+        <is>
+          <t>PG dump file</t>
+        </is>
+      </c>
+      <c r="Q47" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io PG tunnel (port 15432)</t>
+        </is>
+      </c>
       <c r="R47" s="8" t="inlineStr"/>
     </row>
     <row r="48" ht="30" customHeight="1">
@@ -12760,7 +12970,11 @@
           <t>1:00 WITA</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr"/>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Ollama cron window: start/stop Ollama models for test window (01:00-06:05 WITA). Manages model loading/unloading.</t>
+        </is>
+      </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12799,8 +13013,16 @@
       <c r="M50" s="8" t="inlineStr"/>
       <c r="N50" s="8" t="inlineStr"/>
       <c r="O50" s="8" t="inlineStr"/>
-      <c r="P50" s="8" t="inlineStr"/>
-      <c r="Q50" s="8" t="inlineStr"/>
+      <c r="P50" s="8" t="inlineStr">
+        <is>
+          <t>Model load/unload events</t>
+        </is>
+      </c>
+      <c r="Q50" s="8" t="inlineStr">
+        <is>
+          <t>Ollama API</t>
+        </is>
+      </c>
       <c r="R50" s="8" t="inlineStr"/>
     </row>
     <row r="51" ht="30" customHeight="1">
@@ -12824,7 +13046,11 @@
           <t>4:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr"/>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant snapshot (Air): weekly Qdrant cloud snapshot to Tigris S3 backup.</t>
+        </is>
+      </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -12863,8 +13089,16 @@
       <c r="M51" s="8" t="inlineStr"/>
       <c r="N51" s="8" t="inlineStr"/>
       <c r="O51" s="8" t="inlineStr"/>
-      <c r="P51" s="8" t="inlineStr"/>
-      <c r="Q51" s="8" t="inlineStr"/>
+      <c r="P51" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant snapshot on Tigris</t>
+        </is>
+      </c>
+      <c r="Q51" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant API</t>
+        </is>
+      </c>
       <c r="R51" s="8" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
@@ -13268,7 +13502,11 @@
           <t>5:00 WITA</t>
         </is>
       </c>
-      <c r="E57" s="8" t="inlineStr"/>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>MOS TTL cleanup: delete expired memories (where julianday now &gt; created_at + ttl_days).</t>
+        </is>
+      </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -13307,8 +13545,16 @@
       <c r="M57" s="8" t="inlineStr"/>
       <c r="N57" s="8" t="inlineStr"/>
       <c r="O57" s="8" t="inlineStr"/>
-      <c r="P57" s="8" t="inlineStr"/>
-      <c r="Q57" s="8" t="inlineStr"/>
+      <c r="P57" s="8" t="inlineStr">
+        <is>
+          <t>Cleaned memory DB</t>
+        </is>
+      </c>
+      <c r="Q57" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/memory.db</t>
+        </is>
+      </c>
       <c r="R57" s="8" t="inlineStr"/>
     </row>
     <row r="58" ht="30" customHeight="1">
@@ -13484,7 +13730,11 @@
           <t>1:00 WITA Lun</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr"/>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Owner cashout sync: Monday sync of owner weekly cashout data from Fly.io to local spreadsheet.</t>
+        </is>
+      </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -13523,8 +13773,16 @@
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr"/>
       <c r="O60" s="8" t="inlineStr"/>
-      <c r="P60" s="8" t="inlineStr"/>
-      <c r="Q60" s="8" t="inlineStr"/>
+      <c r="P60" s="8" t="inlineStr">
+        <is>
+          <t>Updated cashout data</t>
+        </is>
+      </c>
+      <c r="Q60" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io API, Google Sheets</t>
+        </is>
+      </c>
       <c r="R60" s="8" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
@@ -14077,12 +14335,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>ecosystem-healthcheck</t>
+          <t>daily-ops</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -14092,17 +14350,17 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>8:00 WITA</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Run ecosystem health check. Verify: 1) PostgreSQL is accepting connections (pg_isready). 2) Qdrant is healthy (curl localhost:6333/healthz). 3) Check if Pro is reachable (ssh -o ConnectTimeout=3 pro e</t>
+          <t>Daily morning operations sweep (sequential). Phase 1 - Business Orchestration: review overnight messages, check CRM pipeline health, identify high-priority clients needing follow-up, flag any urgent p</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>qwen3:4b</t>
+          <t>qwen3.5:9b</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -14122,7 +14380,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -14130,32 +14388,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:29</t>
+          <t>2026-04-13 15:29</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>Health report</t>
+          <t>Telegram daily briefing</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Health endpoints</t>
+          <t>CRM, team hours, messages via MCP</t>
         </is>
       </c>
       <c r="R6" s="8" t="inlineStr"/>
@@ -14163,7 +14421,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>fly-health-30m</t>
+          <t>ecosystem-healthcheck</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -14178,12 +14436,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>ogni 30min</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Quick Fly.io health check. Use mcporter call nuzantara-mcp-advanced.check_fly_status. Only report if status is not healthy.</t>
+          <t>Run ecosystem health check. Verify: 1) PostgreSQL is accepting connections (pg_isready). 2) Qdrant is healthy (curl localhost:6333/healthz). 3) Check if Pro is reachable (ssh -o ConnectTimeout=3 pro e</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -14226,7 +14484,7 @@
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 14:54</t>
+          <t>2026-04-13 15:35</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
@@ -14236,12 +14494,12 @@
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Health status</t>
+          <t>Health report</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Fly.io MCP</t>
+          <t>Health endpoints</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr"/>
@@ -14249,12 +14507,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>indexing-daily</t>
+          <t>fly-health-30m</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -14264,22 +14522,22 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>9:00 WITA</t>
+          <t>ogni 30min</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Daily indexing sweep for Google Search Console (sequential). Phase 1 - Articles indexing: submit unindexed intel articles to Google Indexing API (max 200/day quota), update apps/evaluator/articles_ind</t>
+          <t>Quick Fly.io health check. Use mcporter call nuzantara-mcp-advanced.check_fly_status. Only report if status is not healthy.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>qwen3.5:9b</t>
+          <t>qwen3:4b</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>OpenClaw (coder)</t>
+          <t>OpenClaw (main)</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -14294,7 +14552,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -14302,9 +14560,9 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L8" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
@@ -14312,22 +14570,22 @@
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 01:22</t>
+          <t>2026-04-13 15:24</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>Error: All models failed (2): ollama/qwen3:4b: LLM request timed out. (unknown) | google-gemini-cli/</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Submitted URLs to Google</t>
+          <t>Health status</t>
         </is>
       </c>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>GSC API, article list</t>
+          <t>Fly.io MCP</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr"/>
@@ -14335,7 +14593,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>nlm-nb1-daily-refresh</t>
+          <t>indexing-daily</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -14350,12 +14608,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>4:30 WITA</t>
+          <t>9:00 WITA</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Run the NLM NB-1 daily refresh pipeline.  1. Execute:    python3 ~/Desktop/nuzantara/scripts/nlm_nb1_daily_refresh.py  2. Report: how many bundles were updated. 3. If failed, send Telegram alert.</t>
+          <t>Daily indexing sweep for Google Search Console (sequential). Phase 1 - Articles indexing: submit unindexed intel articles to Google Indexing API (max 200/day quota), update apps/evaluator/articles_ind</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -14365,7 +14623,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>OpenClaw (main)</t>
+          <t>OpenClaw (coder)</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -14380,7 +14638,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
@@ -14388,32 +14646,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 20:30</t>
+          <t>2026-04-13 01:22</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Updated NB-1 sources</t>
+          <t>Submitted URLs to Google</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Codebase files</t>
+          <t>GSC API, article list</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr"/>
@@ -14421,12 +14679,12 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>nuz-codebase-audit</t>
+          <t>nlm-nb1-daily-refresh</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -14436,17 +14694,17 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>3:00 WITA Dom</t>
+          <t>4:30 WITA</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Codebase audit for Nuzantara. Do NOT run pytest or any heavy commands. Just do a quick check:  1. Verify the critical import works: source venv/bin/activate &amp;&amp; PYTHONPATH=. python -c 'from backend.app</t>
+          <t>Run the NLM NB-1 daily refresh pipeline.  1. Execute:    python3 ~/Desktop/nuzantara/scripts/nlm_nb1_daily_refresh.py  2. Report: how many bundles were updated. 3. If failed, send Telegram alert.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>qwen3:4b</t>
+          <t>qwen3.5:9b</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -14474,32 +14732,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11 19:00</t>
+          <t>2026-04-12 20:30</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>Audit report</t>
+          <t>Updated NB-1 sources</t>
         </is>
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Git, ruff, pip-audit, coverage</t>
+          <t>Codebase files</t>
         </is>
       </c>
       <c r="R10" s="8" t="inlineStr"/>
@@ -14507,7 +14765,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>nuz-intel-radar</t>
+          <t>nuz-codebase-audit</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -14522,12 +14780,12 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>3:00 WITA Dom</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search the web for the latest Indonesia immigration and business regulation updates from the last 7 days. Focus on: visa policy changes, KBLI updates, PT PMA rules, tax regulation (PPh/PPN). For each </t>
+          <t>Codebase audit for Nuzantara. Do NOT run pytest or any heavy commands. Just do a quick check:  1. Verify the critical import works: source venv/bin/activate &amp;&amp; PYTHONPATH=. python -c 'from backend.app</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -14570,7 +14828,7 @@
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:42</t>
+          <t>2026-04-11 19:00</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
@@ -14580,12 +14838,12 @@
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Intel alerts</t>
+          <t>Audit report</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>News feeds, regulation sites</t>
+          <t>Git, ruff, pip-audit, coverage</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr"/>
@@ -14593,7 +14851,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>nuz-normativa-daily</t>
+          <t>nuz-intel-radar</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -14608,12 +14866,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>7:00 WITA</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>You are the Normativa Pipeline for Nuzantara. Run a DEEP regulatory scan:  1. Search for NEW regulations published in the last 24 hours on:    - bps.go.id (KBLI classifications)    - bkpm.go.id (inves</t>
+          <t xml:space="preserve">Search the web for the latest Indonesia immigration and business regulation updates from the last 7 days. Focus on: visa policy changes, KBLI updates, PT PMA rules, tax regulation (PPh/PPN). For each </t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -14652,26 +14910,26 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:42</t>
+          <t>2026-04-13 15:46</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>cron: job execution timed out</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Regulation change alerts</t>
+          <t>Intel alerts</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>Government sites</t>
+          <t>News feeds, regulation sites</t>
         </is>
       </c>
       <c r="R12" s="8" t="inlineStr"/>
@@ -14679,7 +14937,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>pg-sync-verify</t>
+          <t>nuz-normativa-daily</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -14694,12 +14952,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>5:00 WITA</t>
+          <t>7:00 WITA</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Verify the 03:00 pg-sync completed successfully. Check PostgreSQL logs for errors. Run a basic query (SELECT count(*) FROM clients) to confirm DB is responsive.</t>
+          <t>You are the Normativa Pipeline for Nuzantara. Run a DEEP regulatory scan:  1. Search for NEW regulations published in the last 24 hours on:    - bps.go.id (KBLI classifications)    - bkpm.go.id (inves</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -14742,7 +15000,7 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 09:30</t>
+          <t>2026-04-13 09:42</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
@@ -14752,12 +15010,12 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Verification report</t>
+          <t>Regulation change alerts</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>PG sync output</t>
+          <t>Government sites</t>
         </is>
       </c>
       <c r="R13" s="8" t="inlineStr"/>
@@ -14765,12 +15023,12 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>seo-guardian-observe</t>
+          <t>pg-sync-verify</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -14780,17 +15038,17 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>ogni 40min</t>
+          <t>5:00 WITA</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Run the SEO Guardian observation cycle (Run #25+):  STEP 1 — CHECK SERVICES - Verify backend: curl -s https://nuzantara-rag.fly.dev/health - Verify frontend: curl -I https://balizero.com - Verify llms</t>
+          <t>Verify the 03:00 pg-sync completed successfully. Check PostgreSQL logs for errors. Run a basic query (SELECT count(*) FROM clients) to confirm DB is responsive.</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>qwen3.5:9b</t>
+          <t>qwen3:4b</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -14810,7 +15068,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -14818,32 +15076,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L14" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:01</t>
+          <t>2026-04-13 09:30</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
+          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>Indexed URLs, coverage metrics</t>
+          <t>Verification report</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>GSC API, coverage_state.json</t>
+          <t>PG sync output</t>
         </is>
       </c>
       <c r="R14" s="8" t="inlineStr"/>
@@ -14851,7 +15109,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>seo-guardian-weekly</t>
+          <t>seo-guardian-observe</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -14866,12 +15124,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA Lun</t>
+          <t>ogni 40min</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>You are the SEO Guardian weekly LEARN + REPORT phase.  1. exec: cd ~/Desktop/nuzantara &amp;&amp; source apps/backend-rag/venv/bin/activate &amp;&amp; python3 apps/evaluator/seo_guardian_learn.py 2&gt;&amp;1 2. exec: cd ~/D</t>
+          <t>Run the SEO Guardian observation cycle (Run #25+):  STEP 1 — CHECK SERVICES - Verify backend: curl -s https://nuzantara-rag.fly.dev/health - Verify frontend: curl -I https://balizero.com - Verify llms</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -14910,26 +15168,26 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 00:00</t>
+          <t>2026-04-13 15:01</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>FallbackSummaryError: All models failed (3): ollama/qwen3.5:9b: LLM request timed out. (unknown) | o</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Weekly SEO report, patterns.json</t>
+          <t>Indexed URLs, coverage metrics</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>coverage_state.json, GSC metrics</t>
+          <t>GSC API, coverage_state.json</t>
         </is>
       </c>
       <c r="R15" s="8" t="inlineStr"/>
@@ -14937,12 +15195,12 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>source-enrichment-weekly</t>
+          <t>seo-guardian-weekly</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -14952,17 +15210,17 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>3:00 WITA Dom</t>
+          <t>8:00 WITA Lun</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Run weekly source enrichment batch. Use mcporter call nuzantara-mcp.search_intel query=latest limit=50 to check recent intel, then use mcporter call nuzantara-mcp.publish_intel to publish any enriched</t>
+          <t>You are the SEO Guardian weekly LEARN + REPORT phase.  1. exec: cd ~/Desktop/nuzantara &amp;&amp; source apps/backend-rag/venv/bin/activate &amp;&amp; python3 apps/evaluator/seo_guardian_learn.py 2&gt;&amp;1 2. exec: cd ~/D</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>qwen3:4b</t>
+          <t>qwen3.5:9b</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -14982,7 +15240,7 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K16" s="9" t="inlineStr">
@@ -14990,32 +15248,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11 19:00</t>
+          <t>2026-04-13 00:00</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Updated source registry</t>
+          <t>Weekly SEO report, patterns.json</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>Source registry, web search</t>
+          <t>coverage_state.json, GSC metrics</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr"/>
@@ -15023,12 +15281,12 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>system-doctor</t>
+          <t>source-enrichment-weekly</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -15038,17 +15296,17 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>ogni 4h :0</t>
+          <t>3:00 WITA Dom</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>You are the System Doctor. Diagnose, triage, and fix LOW-risk issues.  Read ~/.openclaw/workspace/autonomous/system-doctor/config.yaml for risk policy.  PHASE 1 — DIAGNOSE (run ALL of these):  1. Back</t>
+          <t>Run weekly source enrichment batch. Use mcporter call nuzantara-mcp.search_intel query=latest limit=50 to check recent intel, then use mcporter call nuzantara-mcp.publish_intel to publish any enriched</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>qwen3.5:9b</t>
+          <t>qwen3:4b</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -15068,7 +15326,7 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
@@ -15076,32 +15334,32 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 12:02</t>
+          <t>2026-04-11 19:00</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
+          <t>LLM request rejected: You're out of extra usage. Add more at claude.ai/settings/usage and keep going</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>Diagnostic report, auto-fixes</t>
+          <t>Updated source registry</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Health endpoints, system state</t>
+          <t>Source registry, web search</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr"/>
@@ -15114,7 +15372,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -15124,17 +15382,17 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>7-19:7,37 WITA</t>
+          <t>ogni 4h :0</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>You are the System Doctor for Nuzantara. Run the collector, read results, act on issues.  STEP 1: python3 scripts/system_doctor.py  STEP 2: Read the JSON output carefully.  STEP 3: - IF escalations ex</t>
+          <t>You are the System Doctor. Diagnose, triage, and fix LOW-risk issues.  Read ~/.openclaw/workspace/autonomous/system-doctor/config.yaml for risk policy.  PHASE 1 — DIAGNOSE (run ALL of these):  1. Back</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>qwen3:4b</t>
+          <t>qwen3.5:9b</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -15168,14 +15426,18 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 11:39</t>
-        </is>
-      </c>
-      <c r="O18" s="8" t="inlineStr"/>
+          <t>2026-04-13 12:02</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
+        </is>
+      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>Diagnostic report, auto-fixes</t>
@@ -15191,12 +15453,12 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>t4-monitor-daily</t>
+          <t>system-doctor</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Air</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -15206,17 +15468,17 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>3:35 WITA</t>
+          <t>7-19:7,37 WITA</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run T4 social media monitor. Execute: bash /Users/nuzantara/Desktop/nuzantara/apps/evaluator/nlm_deep_research/scripts/run_t4_monitor.sh. Check the log at ~/.openclaw/logs/t4_monitor.log for results. </t>
+          <t>You are the System Doctor for Nuzantara. Run the collector, read results, act on issues.  STEP 1: python3 scripts/system_doctor.py  STEP 2: Read the JSON output carefully.  STEP 3: - IF escalations ex</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>qwen3.5:9b</t>
+          <t>qwen3:4b</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -15236,7 +15498,7 @@
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LOCAL</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
@@ -15244,32 +15506,28 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 19:37</t>
-        </is>
-      </c>
-      <c r="O19" s="8" t="inlineStr">
-        <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
-        </is>
-      </c>
+          <t>2026-04-13 11:39</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr"/>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>Social media report</t>
+          <t>Diagnostic report, auto-fixes</t>
         </is>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>T4 monitor script output</t>
+          <t>Health endpoints, system state</t>
         </is>
       </c>
       <c r="R19" s="8" t="inlineStr"/>
@@ -15277,7 +15535,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>tech-orchestrator</t>
+          <t>t4-monitor-daily</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -15292,12 +15550,12 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>ogni 4h</t>
+          <t>3:35 WITA</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GUARDRAILS (controlla PRIMA di qualsiasi azione):  1. BLACKOUT WINDOW: exec: hour=$(TZ='Asia/Makassar' date +%H); if [ "$hour" -ge 0 ] &amp;&amp; [ "$hour" -lt 3 ]; then echo 'BLACKOUT_00-03_WITA_SKIP'; exit </t>
+          <t xml:space="preserve">Run T4 social media monitor. Execute: bash /Users/nuzantara/Desktop/nuzantara/apps/evaluator/nlm_deep_research/scripts/run_t4_monitor.sh. Check the log at ~/.openclaw/logs/t4_monitor.log for results. </t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -15322,7 +15580,7 @@
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">
@@ -15330,17 +15588,17 @@
           <t>failed</t>
         </is>
       </c>
-      <c r="L20" s="9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 13:00</t>
+          <t>2026-04-12 19:37</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
@@ -15350,12 +15608,12 @@
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>Deploy decision, issue list</t>
+          <t>Social media report</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Git diff, fly status, Core Guardian output</t>
+          <t>T4 monitor script output</t>
         </is>
       </c>
       <c r="R20" s="8" t="inlineStr"/>
@@ -15363,7 +15621,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>weekly-dep-audit</t>
+          <t>tech-orchestrator</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -15378,12 +15636,12 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>3:30 WITA Lun</t>
+          <t>ogni 4h</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Run weekly dependency audit with auto-patch for safe (patch-only) upgrades.  PHASE 1 — AUDIT: 1. mcporter call nuzantara-mcp-advanced.check_deployment_readiness  2. Python outdated:    exec: source .v</t>
+          <t xml:space="preserve">GUARDRAILS (controlla PRIMA di qualsiasi azione):  1. BLACKOUT WINDOW: exec: hour=$(TZ='Asia/Makassar' date +%H); if [ "$hour" -ge 0 ] &amp;&amp; [ "$hour" -lt 3 ]; then echo 'BLACKOUT_00-03_WITA_SKIP'; exit </t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -15422,11 +15680,11 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 19:33</t>
+          <t>2026-04-13 13:00</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
@@ -15436,12 +15694,12 @@
       </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
-          <t>Audit report, patched deps</t>
+          <t>Deploy decision, issue list</t>
         </is>
       </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>pyproject.toml, pip-audit</t>
+          <t>Git diff, fly status, Core Guardian output</t>
         </is>
       </c>
       <c r="R21" s="8" t="inlineStr"/>
@@ -15449,7 +15707,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>weekly-review</t>
+          <t>weekly-dep-audit</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -15464,12 +15722,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>9:00 WITA Lun</t>
+          <t>3:30 WITA Lun</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Weekly Monday review — business KPIs + technical quality (sequential). Phase 1 - Business Report: summarize week revenue and invoices, new clients onboarded, practice completions, team hours, complian</t>
+          <t>Run weekly dependency audit with auto-patch for safe (patch-only) upgrades.  PHASE 1 — AUDIT: 1. mcporter call nuzantara-mcp-advanced.check_deployment_readiness  2. Python outdated:    exec: source .v</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -15508,26 +15766,26 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 01:39</t>
+          <t>2026-04-12 19:33</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: ⚠️ Cloud Code</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
-          <t>Telegram weekly report</t>
+          <t>Audit report, patched deps</t>
         </is>
       </c>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>CRM, code quality, Fly.io metrics via MCP</t>
+          <t>pyproject.toml, pip-audit</t>
         </is>
       </c>
       <c r="R22" s="8" t="inlineStr"/>
@@ -15535,7 +15793,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>cell-weekly-report</t>
+          <t>weekly-review</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -15550,12 +15808,12 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA Dom</t>
+          <t>9:00 WITA Lun</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>PLACEHOLDER — Cell organism weekly report. Task empty.</t>
+          <t>Weekly Monday review — business KPIs + technical quality (sequential). Phase 1 - Business Report: summarize week revenue and invoices, new clients onboarded, practice completions, team hours, complian</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -15580,48 +15838,48 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K23" s="10" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="L23" s="11" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
+          <t>LOCAL</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>2026-04-12 00:04</t>
-        </is>
-      </c>
-      <c r="O23" s="8" t="inlineStr"/>
+          <t>2026-04-13 01:39</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="inlineStr">
+        <is>
+          <t>FallbackSummaryError: All models failed (3): google-gemini-cli/gemini-3-flash-preview: LLM request t</t>
+        </is>
+      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Telegram weekly report</t>
         </is>
       </c>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R23" s="8" t="inlineStr">
-        <is>
-          <t>Skipped: empty task.</t>
-        </is>
-      </c>
+          <t>CRM, code quality, Fly.io metrics via MCP</t>
+        </is>
+      </c>
+      <c r="R23" s="8" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>daily-ops</t>
+          <t>cell-weekly-report</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -15636,12 +15894,12 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>8:00 WITA</t>
+          <t>8:00 WITA Dom</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Daily morning operations sweep (sequential). Phase 1 - Business Orchestration: review overnight messages, check CRM pipeline health, identify high-priority clients needing follow-up, flag any urgent p</t>
+          <t>PLACEHOLDER — Cell organism weekly report. Task empty.</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -15666,37 +15924,43 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>LOCAL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="L24" s="11" t="inlineStr">
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="L24" s="10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="M24" s="8" t="inlineStr"/>
+      <c r="M24" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:07</t>
+          <t>2026-04-12 00:04</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr"/>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>Telegram daily briefing</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>CRM, team hours, messages via MCP</t>
-        </is>
-      </c>
-      <c r="R24" s="8" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R24" s="8" t="inlineStr">
+        <is>
+          <t>Skipped: empty task.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
@@ -15749,7 +16013,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K25" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -15829,7 +16093,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
+      <c r="K26" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -15909,12 +16173,12 @@
           <t>LOCAL</t>
         </is>
       </c>
-      <c r="K27" s="11" t="inlineStr">
+      <c r="K27" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="L27" s="11" t="inlineStr">
+      <c r="L27" s="10" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -15989,17 +16253,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K28" s="10" t="inlineStr">
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M28" s="8" t="inlineStr"/>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 17:10</t>
@@ -16073,17 +16339,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K29" s="10" t="inlineStr">
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr"/>
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:50</t>
@@ -16157,17 +16425,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K30" s="10" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M30" s="8" t="inlineStr"/>
+      <c r="L30" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M30" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:45</t>
@@ -16241,17 +16511,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K31" s="10" t="inlineStr">
+      <c r="K31" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M31" s="8" t="inlineStr"/>
+      <c r="L31" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:20</t>
@@ -16325,17 +16597,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K32" s="10" t="inlineStr">
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L32" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M32" s="8" t="inlineStr"/>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M32" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:35</t>
@@ -16409,17 +16683,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K33" s="10" t="inlineStr">
+      <c r="K33" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M33" s="8" t="inlineStr"/>
+      <c r="L33" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:30</t>
@@ -16493,17 +16769,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K34" s="10" t="inlineStr">
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L34" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M34" s="8" t="inlineStr"/>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:40</t>
@@ -16577,17 +16855,19 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K35" s="10" t="inlineStr">
+      <c r="K35" s="11" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
       </c>
-      <c r="L35" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M35" s="8" t="inlineStr"/>
+      <c r="L35" s="10" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
           <t>2026-04-12 18:47</t>
@@ -16661,7 +16941,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="K36" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -16741,7 +17021,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="K37" s="11" t="inlineStr">
+      <c r="K37" s="10" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
@@ -20619,7 +20899,11 @@
           <t>3:30 WITA giorno 1,15</t>
         </is>
       </c>
-      <c r="E89" s="8" t="inlineStr"/>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>Orphan crontab entry — incomplete script reference. Likely a broken entry.</t>
+        </is>
+      </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20660,7 +20944,11 @@
       <c r="O89" s="8" t="inlineStr"/>
       <c r="P89" s="8" t="inlineStr"/>
       <c r="Q89" s="8" t="inlineStr"/>
-      <c r="R89" s="8" t="inlineStr"/>
+      <c r="R89" s="8" t="inlineStr">
+        <is>
+          <t>AUDIT: remove or fix in crontab</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="8" t="inlineStr">
@@ -20683,7 +20971,11 @@
           <t>7:30 WITA</t>
         </is>
       </c>
-      <c r="E90" s="8" t="inlineStr"/>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>Auto practice creator: POST to Fly.io API to auto-create practices for expiring visas at T-60 days.</t>
+        </is>
+      </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20722,8 +21014,16 @@
       <c r="M90" s="8" t="inlineStr"/>
       <c r="N90" s="8" t="inlineStr"/>
       <c r="O90" s="8" t="inlineStr"/>
-      <c r="P90" s="8" t="inlineStr"/>
-      <c r="Q90" s="8" t="inlineStr"/>
+      <c r="P90" s="8" t="inlineStr">
+        <is>
+          <t>New CRM practices</t>
+        </is>
+      </c>
+      <c r="Q90" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R90" s="8" t="inlineStr"/>
     </row>
     <row r="91" ht="30" customHeight="1">
@@ -20747,7 +21047,11 @@
           <t>0:00 WITA</t>
         </is>
       </c>
-      <c r="E91" s="8" t="inlineStr"/>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>All notifiers: trigger visa expiry, unpaid invoices, stale practice alerts via backend API.</t>
+        </is>
+      </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20786,8 +21090,16 @@
       <c r="M91" s="8" t="inlineStr"/>
       <c r="N91" s="8" t="inlineStr"/>
       <c r="O91" s="8" t="inlineStr"/>
-      <c r="P91" s="8" t="inlineStr"/>
-      <c r="Q91" s="8" t="inlineStr"/>
+      <c r="P91" s="8" t="inlineStr">
+        <is>
+          <t>Client alerts (WhatsApp/email/Telegram)</t>
+        </is>
+      </c>
+      <c r="Q91" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R91" s="8" t="inlineStr"/>
     </row>
     <row r="92" ht="30" customHeight="1">
@@ -20811,7 +21123,11 @@
           <t>0:05 WITA</t>
         </is>
       </c>
-      <c r="E92" s="8" t="inlineStr"/>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Birthday notifier: send birthday greetings to clients via backend API.</t>
+        </is>
+      </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20850,8 +21166,16 @@
       <c r="M92" s="8" t="inlineStr"/>
       <c r="N92" s="8" t="inlineStr"/>
       <c r="O92" s="8" t="inlineStr"/>
-      <c r="P92" s="8" t="inlineStr"/>
-      <c r="Q92" s="8" t="inlineStr"/>
+      <c r="P92" s="8" t="inlineStr">
+        <is>
+          <t>Birthday greeting messages</t>
+        </is>
+      </c>
+      <c r="Q92" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R92" s="8" t="inlineStr"/>
     </row>
     <row r="93" ht="30" customHeight="1">
@@ -20875,7 +21199,11 @@
           <t>ogni 15min</t>
         </is>
       </c>
-      <c r="E93" s="8" t="inlineStr"/>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>Welcome pending: send welcome emails to new clients after 30min delay. Every 15min.</t>
+        </is>
+      </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20914,8 +21242,16 @@
       <c r="M93" s="8" t="inlineStr"/>
       <c r="N93" s="8" t="inlineStr"/>
       <c r="O93" s="8" t="inlineStr"/>
-      <c r="P93" s="8" t="inlineStr"/>
-      <c r="Q93" s="8" t="inlineStr"/>
+      <c r="P93" s="8" t="inlineStr">
+        <is>
+          <t>Welcome emails</t>
+        </is>
+      </c>
+      <c r="Q93" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io backend API</t>
+        </is>
+      </c>
       <c r="R93" s="8" t="inlineStr"/>
     </row>
     <row r="94" ht="30" customHeight="1">
@@ -20939,7 +21275,11 @@
           <t>2:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E94" s="8" t="inlineStr"/>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>Weekly audit trail cleanup: prune old audit log entries on Air.</t>
+        </is>
+      </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -20978,8 +21318,16 @@
       <c r="M94" s="8" t="inlineStr"/>
       <c r="N94" s="8" t="inlineStr"/>
       <c r="O94" s="8" t="inlineStr"/>
-      <c r="P94" s="8" t="inlineStr"/>
-      <c r="Q94" s="8" t="inlineStr"/>
+      <c r="P94" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q94" s="8" t="inlineStr">
+        <is>
+          <t>Audit log files</t>
+        </is>
+      </c>
       <c r="R94" s="8" t="inlineStr"/>
     </row>
     <row r="95" ht="30" customHeight="1">
@@ -21383,7 +21731,11 @@
           <t>3:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E100" s="8" t="inlineStr"/>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>Weekly conversation trainer: trigger conversation-trainer OpenClaw job via cron-runner wrapper. Extracts patterns from recent chats.</t>
+        </is>
+      </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21422,8 +21774,16 @@
       <c r="M100" s="8" t="inlineStr"/>
       <c r="N100" s="8" t="inlineStr"/>
       <c r="O100" s="8" t="inlineStr"/>
-      <c r="P100" s="8" t="inlineStr"/>
-      <c r="Q100" s="8" t="inlineStr"/>
+      <c r="P100" s="8" t="inlineStr">
+        <is>
+          <t>Training patterns</t>
+        </is>
+      </c>
+      <c r="Q100" s="8" t="inlineStr">
+        <is>
+          <t>Recent conversations, OpenClaw gateway</t>
+        </is>
+      </c>
       <c r="R100" s="8" t="inlineStr"/>
     </row>
     <row r="101" ht="30" customHeight="1">
@@ -21447,7 +21807,11 @@
           <t>4:00 WITA</t>
         </is>
       </c>
-      <c r="E101" s="8" t="inlineStr"/>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>MOS daily backup: copy memory.db to timestamped backup file.</t>
+        </is>
+      </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21486,8 +21850,16 @@
       <c r="M101" s="8" t="inlineStr"/>
       <c r="N101" s="8" t="inlineStr"/>
       <c r="O101" s="8" t="inlineStr"/>
-      <c r="P101" s="8" t="inlineStr"/>
-      <c r="Q101" s="8" t="inlineStr"/>
+      <c r="P101" s="8" t="inlineStr">
+        <is>
+          <t>Memory DB backup</t>
+        </is>
+      </c>
+      <c r="Q101" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/memory.db</t>
+        </is>
+      </c>
       <c r="R101" s="8" t="inlineStr"/>
     </row>
     <row r="102" ht="30" customHeight="1">
@@ -21511,7 +21883,11 @@
           <t>23:00 WITA</t>
         </is>
       </c>
-      <c r="E102" s="8" t="inlineStr"/>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>CRM automation engine: quality checks, document follow-up, renewal processing. Runs nightly on Air.</t>
+        </is>
+      </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21550,8 +21926,16 @@
       <c r="M102" s="8" t="inlineStr"/>
       <c r="N102" s="8" t="inlineStr"/>
       <c r="O102" s="8" t="inlineStr"/>
-      <c r="P102" s="8" t="inlineStr"/>
-      <c r="Q102" s="8" t="inlineStr"/>
+      <c r="P102" s="8" t="inlineStr">
+        <is>
+          <t>CRM updates, follow-up tasks</t>
+        </is>
+      </c>
+      <c r="Q102" s="8" t="inlineStr">
+        <is>
+          <t>Backend API CRM data</t>
+        </is>
+      </c>
       <c r="R102" s="8" t="inlineStr"/>
     </row>
     <row r="103" ht="30" customHeight="1">
@@ -21575,7 +21959,11 @@
           <t>23:00 WITA</t>
         </is>
       </c>
-      <c r="E103" s="8" t="inlineStr"/>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>Cron wrapper: universal wrapper that adds logging, locking, timeout, and Telegram alerts to any cron script.</t>
+        </is>
+      </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21614,8 +22002,16 @@
       <c r="M103" s="8" t="inlineStr"/>
       <c r="N103" s="8" t="inlineStr"/>
       <c r="O103" s="8" t="inlineStr"/>
-      <c r="P103" s="8" t="inlineStr"/>
-      <c r="Q103" s="8" t="inlineStr"/>
+      <c r="P103" s="8" t="inlineStr">
+        <is>
+          <t>Structured logs, state files</t>
+        </is>
+      </c>
+      <c r="Q103" s="8" t="inlineStr">
+        <is>
+          <t>Wrapped script output</t>
+        </is>
+      </c>
       <c r="R103" s="8" t="inlineStr"/>
     </row>
     <row r="104" ht="30" customHeight="1">
@@ -21791,7 +22187,11 @@
           <t>ogni 4min</t>
         </is>
       </c>
-      <c r="E106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>NLM bridge state writer: write heartbeat JSON for Sentinel to monitor NLM bridge daemon.</t>
+        </is>
+      </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21830,8 +22230,16 @@
       <c r="M106" s="8" t="inlineStr"/>
       <c r="N106" s="8" t="inlineStr"/>
       <c r="O106" s="8" t="inlineStr"/>
-      <c r="P106" s="8" t="inlineStr"/>
-      <c r="Q106" s="8" t="inlineStr"/>
+      <c r="P106" s="8" t="inlineStr">
+        <is>
+          <t>State JSON for Sentinel</t>
+        </is>
+      </c>
+      <c r="Q106" s="8" t="inlineStr">
+        <is>
+          <t>System clock</t>
+        </is>
+      </c>
       <c r="R106" s="8" t="inlineStr"/>
     </row>
     <row r="107" ht="30" customHeight="1">
@@ -21931,7 +22339,11 @@
           <t>5:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E108" s="8" t="inlineStr"/>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>MOS backup pruning: delete memory backups older than 30 days.</t>
+        </is>
+      </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -21970,8 +22382,16 @@
       <c r="M108" s="8" t="inlineStr"/>
       <c r="N108" s="8" t="inlineStr"/>
       <c r="O108" s="8" t="inlineStr"/>
-      <c r="P108" s="8" t="inlineStr"/>
-      <c r="Q108" s="8" t="inlineStr"/>
+      <c r="P108" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q108" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/backups/</t>
+        </is>
+      </c>
       <c r="R108" s="8" t="inlineStr"/>
     </row>
     <row r="109" ht="30" customHeight="1">
@@ -22223,7 +22643,11 @@
           <t>3:20 WITA</t>
         </is>
       </c>
-      <c r="E112" s="8" t="inlineStr"/>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>Fly PG backup (Air): pg_dump from Fly.io PG tunnel to local backup. Separate from Pro fly-backup.sh.</t>
+        </is>
+      </c>
       <c r="F112" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -22262,8 +22686,16 @@
       <c r="M112" s="8" t="inlineStr"/>
       <c r="N112" s="8" t="inlineStr"/>
       <c r="O112" s="8" t="inlineStr"/>
-      <c r="P112" s="8" t="inlineStr"/>
-      <c r="Q112" s="8" t="inlineStr"/>
+      <c r="P112" s="8" t="inlineStr">
+        <is>
+          <t>PG dump file</t>
+        </is>
+      </c>
+      <c r="Q112" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io PG tunnel (port 15432)</t>
+        </is>
+      </c>
       <c r="R112" s="8" t="inlineStr"/>
     </row>
     <row r="113" ht="30" customHeight="1">
@@ -22515,7 +22947,11 @@
           <t>2:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E116" s="8" t="inlineStr"/>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t>Weekly KG builder: trigger knowledge-graph-builder OpenClaw job via cron-runner wrapper. Ingests entities into Neo4j.</t>
+        </is>
+      </c>
       <c r="F116" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -22554,8 +22990,16 @@
       <c r="M116" s="8" t="inlineStr"/>
       <c r="N116" s="8" t="inlineStr"/>
       <c r="O116" s="8" t="inlineStr"/>
-      <c r="P116" s="8" t="inlineStr"/>
-      <c r="Q116" s="8" t="inlineStr"/>
+      <c r="P116" s="8" t="inlineStr">
+        <is>
+          <t>KG entities (Neo4j)</t>
+        </is>
+      </c>
+      <c r="Q116" s="8" t="inlineStr">
+        <is>
+          <t>Conversation data, OpenClaw gateway</t>
+        </is>
+      </c>
       <c r="R116" s="8" t="inlineStr"/>
     </row>
     <row r="117" ht="30" customHeight="1">
@@ -22731,7 +23175,11 @@
           <t>3:30 WITA giorno 1,15</t>
         </is>
       </c>
-      <c r="E119" s="8" t="inlineStr"/>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>Cache cleanup: npm + pip + brew cache purge. Runs 1st and 15th of each month.</t>
+        </is>
+      </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -22770,8 +23218,16 @@
       <c r="M119" s="8" t="inlineStr"/>
       <c r="N119" s="8" t="inlineStr"/>
       <c r="O119" s="8" t="inlineStr"/>
-      <c r="P119" s="8" t="inlineStr"/>
-      <c r="Q119" s="8" t="inlineStr"/>
+      <c r="P119" s="8" t="inlineStr">
+        <is>
+          <t>Freed disk space</t>
+        </is>
+      </c>
+      <c r="Q119" s="8" t="inlineStr">
+        <is>
+          <t>npm/pip/brew caches</t>
+        </is>
+      </c>
       <c r="R119" s="8" t="inlineStr"/>
     </row>
     <row r="120" ht="30" customHeight="1">
@@ -22947,7 +23403,11 @@
           <t>1:00 WITA</t>
         </is>
       </c>
-      <c r="E122" s="8" t="inlineStr"/>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>Ollama cron window: start/stop Ollama models for test window (01:00-06:05 WITA). Manages model loading/unloading.</t>
+        </is>
+      </c>
       <c r="F122" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -22986,8 +23446,16 @@
       <c r="M122" s="8" t="inlineStr"/>
       <c r="N122" s="8" t="inlineStr"/>
       <c r="O122" s="8" t="inlineStr"/>
-      <c r="P122" s="8" t="inlineStr"/>
-      <c r="Q122" s="8" t="inlineStr"/>
+      <c r="P122" s="8" t="inlineStr">
+        <is>
+          <t>Model load/unload events</t>
+        </is>
+      </c>
+      <c r="Q122" s="8" t="inlineStr">
+        <is>
+          <t>Ollama API</t>
+        </is>
+      </c>
       <c r="R122" s="8" t="inlineStr"/>
     </row>
     <row r="123" ht="30" customHeight="1">
@@ -23087,7 +23555,11 @@
           <t>4:00 WITA Dom</t>
         </is>
       </c>
-      <c r="E124" s="8" t="inlineStr"/>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant snapshot (Air): weekly Qdrant cloud snapshot to Tigris S3 backup.</t>
+        </is>
+      </c>
       <c r="F124" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -23126,8 +23598,16 @@
       <c r="M124" s="8" t="inlineStr"/>
       <c r="N124" s="8" t="inlineStr"/>
       <c r="O124" s="8" t="inlineStr"/>
-      <c r="P124" s="8" t="inlineStr"/>
-      <c r="Q124" s="8" t="inlineStr"/>
+      <c r="P124" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant snapshot on Tigris</t>
+        </is>
+      </c>
+      <c r="Q124" s="8" t="inlineStr">
+        <is>
+          <t>Qdrant API</t>
+        </is>
+      </c>
       <c r="R124" s="8" t="inlineStr"/>
     </row>
     <row r="125" ht="30" customHeight="1">
@@ -25583,7 +26063,11 @@
           <t>5:00 WITA</t>
         </is>
       </c>
-      <c r="E157" s="8" t="inlineStr"/>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>MOS TTL cleanup: delete expired memories (where julianday now &gt; created_at + ttl_days).</t>
+        </is>
+      </c>
       <c r="F157" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -25622,8 +26106,16 @@
       <c r="M157" s="8" t="inlineStr"/>
       <c r="N157" s="8" t="inlineStr"/>
       <c r="O157" s="8" t="inlineStr"/>
-      <c r="P157" s="8" t="inlineStr"/>
-      <c r="Q157" s="8" t="inlineStr"/>
+      <c r="P157" s="8" t="inlineStr">
+        <is>
+          <t>Cleaned memory DB</t>
+        </is>
+      </c>
+      <c r="Q157" s="8" t="inlineStr">
+        <is>
+          <t>~/.claude/memory.db</t>
+        </is>
+      </c>
       <c r="R157" s="8" t="inlineStr"/>
     </row>
     <row r="158" ht="30" customHeight="1">
@@ -26027,7 +26519,11 @@
           <t>1:00 WITA Lun</t>
         </is>
       </c>
-      <c r="E163" s="8" t="inlineStr"/>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>Owner cashout sync: Monday sync of owner weekly cashout data from Fly.io to local spreadsheet.</t>
+        </is>
+      </c>
       <c r="F163" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -26066,8 +26562,16 @@
       <c r="M163" s="8" t="inlineStr"/>
       <c r="N163" s="8" t="inlineStr"/>
       <c r="O163" s="8" t="inlineStr"/>
-      <c r="P163" s="8" t="inlineStr"/>
-      <c r="Q163" s="8" t="inlineStr"/>
+      <c r="P163" s="8" t="inlineStr">
+        <is>
+          <t>Updated cashout data</t>
+        </is>
+      </c>
+      <c r="Q163" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io API, Google Sheets</t>
+        </is>
+      </c>
       <c r="R163" s="8" t="inlineStr"/>
     </row>
     <row r="164" ht="30" customHeight="1">
@@ -26167,7 +26671,11 @@
           <t>ogni ora :0</t>
         </is>
       </c>
-      <c r="E165" s="8" t="inlineStr"/>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>Pro heartbeat: write timestamp locally + push to Air via SSH. Hourly dead-man switch.</t>
+        </is>
+      </c>
       <c r="F165" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -26206,8 +26714,16 @@
       <c r="M165" s="8" t="inlineStr"/>
       <c r="N165" s="8" t="inlineStr"/>
       <c r="O165" s="8" t="inlineStr"/>
-      <c r="P165" s="8" t="inlineStr"/>
-      <c r="Q165" s="8" t="inlineStr"/>
+      <c r="P165" s="8" t="inlineStr">
+        <is>
+          <t>Heartbeat file on both nodes</t>
+        </is>
+      </c>
+      <c r="Q165" s="8" t="inlineStr">
+        <is>
+          <t>SSH to Air</t>
+        </is>
+      </c>
       <c r="R165" s="8" t="inlineStr"/>
     </row>
     <row r="166" ht="30" customHeight="1">

</xml_diff>

<commit_message>
feat: add Backend Services sheet + fill all empty columns
New "Backend" sheet: 11 asyncio background loops running inside
FastAPI on Fly.io (Olympus heartbeat/pulse, Compliance Monitor,
Practice Status Listener, X Monitor, Health Monitor, Alert Digest,
EventBus, Team Timesheet, Autonomous Scheduler).

Total: 176 automations (Pro 105 + Air 60 + Backend 11).

Column fill rates: Sistema 99%, Descrizione 100%, Monitorato 100%,
Stato 100%, Produce 94%, Consuma 94%.

Also: launchctl status detection for LaunchAgents, default
monitored_by for all non-Sentinel jobs, system classification
with underscore/dash normalization.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/automations-inventory.xlsx
+++ b/docs/automations-inventory.xlsx
@@ -10,12 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pro" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Air" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pro'!$A$1:$S$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Air'!$A$1:$S$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backend'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'All'!$A$1:$S$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -592,7 +594,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-14 00:09 WITA</t>
+          <t>Generated: 2026-04-14 00:16 WITA</t>
         </is>
       </c>
     </row>
@@ -14794,7 +14796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S166"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14918,6 +14920,1038 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
+          <t>alert_service_digest</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>ogni ora (next hour boundary)</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Alert digest: hourly aggregation of all alerts, sends condensed summary instead of individual notifications to prevent alert fatigue.</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr"/>
+      <c r="O2" s="8" t="inlineStr"/>
+      <c r="P2" s="8" t="inlineStr"/>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>Aggregated alert digest</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t>Individual alert events</t>
+        </is>
+      </c>
+      <c r="S2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>autonomous_scheduler</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (per remaining tasks)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr"/>
+      <c r="O3" s="8" t="inlineStr"/>
+      <c r="P3" s="8" t="inlineStr"/>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>Self-healing actions</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>Service health status</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven, ping 30s)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr"/>
+      <c r="O4" s="8" t="inlineStr"/>
+      <c r="P4" s="8" t="inlineStr"/>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>Routed events to subscribers</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>Redis Streams (all channels)</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>ogni 60s</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Self (top-level monitor)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr"/>
+      <c r="O5" s="8" t="inlineStr"/>
+      <c r="P5" s="8" t="inlineStr"/>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>Service health status, degradation alerts</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>All internal service health endpoints</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr"/>
+      <c r="O6" s="8" t="inlineStr"/>
+      <c r="P6" s="8" t="inlineStr"/>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>Health metrics, PG stats</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>PostgreSQL pg_stat_statements</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>ogni 6h</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr"/>
+      <c r="O7" s="8" t="inlineStr"/>
+      <c r="P7" s="8" t="inlineStr"/>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>olympus_insights, PulseAction, alerts</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>practice_status_listener</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr"/>
+      <c r="O8" s="8" t="inlineStr"/>
+      <c r="P8" s="8" t="inlineStr"/>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>Practice state change events</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>Redis pub/sub practice_status channel</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>proactive_compliance_monitor</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>ogni 24h (86400s)</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr"/>
+      <c r="O9" s="8" t="inlineStr"/>
+      <c r="P9" s="8" t="inlineStr"/>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr"/>
+      <c r="O10" s="8" t="inlineStr"/>
+      <c r="P10" s="8" t="inlineStr"/>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>Auto-closed timesheet sessions</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>work_sessions table</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr"/>
+      <c r="O11" s="8" t="inlineStr"/>
+      <c r="P11" s="8" t="inlineStr"/>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L12" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr"/>
+      <c r="O12" s="8" t="inlineStr"/>
+      <c r="P12" s="8" t="inlineStr"/>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>Twitter match entries</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>Twitter API v2 search/recent</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>CRC broken — X API access issues</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S177"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="35" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Macchina</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Usa LLM</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Interfaccia LLM</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Monitorato da</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Critico</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Repair Scope</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Stato</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Circuit Breaker</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Errori</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Ultimo Run</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Ultimo Errore</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Consuma</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
           <t>client-health-monitor</t>
         </is>
       </c>
@@ -28561,6 +29595,905 @@
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
+    </row>
+    <row r="167" ht="30" customHeight="1">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>alert_service_digest</t>
+        </is>
+      </c>
+      <c r="B167" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>ogni ora (next hour boundary)</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="inlineStr">
+        <is>
+          <t>Alert digest: hourly aggregation of all alerts, sends condensed summary instead of individual notifications to prevent alert fatigue.</t>
+        </is>
+      </c>
+      <c r="G167" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H167" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I167" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J167" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K167" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L167" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M167" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N167" s="8" t="inlineStr"/>
+      <c r="O167" s="8" t="inlineStr"/>
+      <c r="P167" s="8" t="inlineStr"/>
+      <c r="Q167" s="8" t="inlineStr">
+        <is>
+          <t>Aggregated alert digest</t>
+        </is>
+      </c>
+      <c r="R167" s="8" t="inlineStr">
+        <is>
+          <t>Individual alert events</t>
+        </is>
+      </c>
+      <c r="S167" s="8" t="inlineStr"/>
+    </row>
+    <row r="168" ht="30" customHeight="1">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
+          <t>autonomous_scheduler</t>
+        </is>
+      </c>
+      <c r="B168" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D168" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E168" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (per remaining tasks)</t>
+        </is>
+      </c>
+      <c r="F168" s="8" t="inlineStr">
+        <is>
+          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
+        </is>
+      </c>
+      <c r="G168" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H168" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I168" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J168" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K168" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L168" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M168" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N168" s="8" t="inlineStr"/>
+      <c r="O168" s="8" t="inlineStr"/>
+      <c r="P168" s="8" t="inlineStr"/>
+      <c r="Q168" s="8" t="inlineStr">
+        <is>
+          <t>Self-healing actions</t>
+        </is>
+      </c>
+      <c r="R168" s="8" t="inlineStr">
+        <is>
+          <t>Service health status</t>
+        </is>
+      </c>
+      <c r="S168" s="8" t="inlineStr">
+        <is>
+          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="30" customHeight="1">
+      <c r="A169" s="8" t="inlineStr">
+        <is>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C169" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E169" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven, ping 30s)</t>
+        </is>
+      </c>
+      <c r="F169" s="8" t="inlineStr">
+        <is>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+        </is>
+      </c>
+      <c r="G169" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H169" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I169" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J169" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K169" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L169" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M169" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N169" s="8" t="inlineStr"/>
+      <c r="O169" s="8" t="inlineStr"/>
+      <c r="P169" s="8" t="inlineStr"/>
+      <c r="Q169" s="8" t="inlineStr">
+        <is>
+          <t>Routed events to subscribers</t>
+        </is>
+      </c>
+      <c r="R169" s="8" t="inlineStr">
+        <is>
+          <t>Redis Streams (all channels)</t>
+        </is>
+      </c>
+      <c r="S169" s="8" t="inlineStr"/>
+    </row>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E170" s="8" t="inlineStr">
+        <is>
+          <t>ogni 60s</t>
+        </is>
+      </c>
+      <c r="F170" s="8" t="inlineStr">
+        <is>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+        </is>
+      </c>
+      <c r="G170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I170" s="8" t="inlineStr">
+        <is>
+          <t>Self (top-level monitor)</t>
+        </is>
+      </c>
+      <c r="J170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L170" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M170" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N170" s="8" t="inlineStr"/>
+      <c r="O170" s="8" t="inlineStr"/>
+      <c r="P170" s="8" t="inlineStr"/>
+      <c r="Q170" s="8" t="inlineStr">
+        <is>
+          <t>Service health status, degradation alerts</t>
+        </is>
+      </c>
+      <c r="R170" s="8" t="inlineStr">
+        <is>
+          <t>All internal service health endpoints</t>
+        </is>
+      </c>
+      <c r="S170" s="8" t="inlineStr"/>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="A171" s="8" t="inlineStr">
+        <is>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B171" s="19" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E171" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F171" s="8" t="inlineStr">
+        <is>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+        </is>
+      </c>
+      <c r="G171" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H171" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I171" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J171" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K171" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L171" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M171" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N171" s="8" t="inlineStr"/>
+      <c r="O171" s="8" t="inlineStr"/>
+      <c r="P171" s="8" t="inlineStr"/>
+      <c r="Q171" s="8" t="inlineStr">
+        <is>
+          <t>Health metrics, PG stats</t>
+        </is>
+      </c>
+      <c r="R171" s="8" t="inlineStr">
+        <is>
+          <t>PostgreSQL pg_stat_statements</t>
+        </is>
+      </c>
+      <c r="S171" s="8" t="inlineStr"/>
+    </row>
+    <row r="172" ht="30" customHeight="1">
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B172" s="19" t="inlineStr">
+        <is>
+          <t>Olympus</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>ogni 6h</t>
+        </is>
+      </c>
+      <c r="F172" s="8" t="inlineStr">
+        <is>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+        </is>
+      </c>
+      <c r="G172" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H172" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I172" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J172" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K172" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L172" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M172" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N172" s="8" t="inlineStr"/>
+      <c r="O172" s="8" t="inlineStr"/>
+      <c r="P172" s="8" t="inlineStr"/>
+      <c r="Q172" s="8" t="inlineStr">
+        <is>
+          <t>olympus_insights, PulseAction, alerts</t>
+        </is>
+      </c>
+      <c r="R172" s="8" t="inlineStr">
+        <is>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+        </is>
+      </c>
+      <c r="S172" s="8" t="inlineStr"/>
+    </row>
+    <row r="173" ht="30" customHeight="1">
+      <c r="A173" s="8" t="inlineStr">
+        <is>
+          <t>practice_status_listener</t>
+        </is>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E173" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven)</t>
+        </is>
+      </c>
+      <c r="F173" s="8" t="inlineStr">
+        <is>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+        </is>
+      </c>
+      <c r="G173" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H173" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J173" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K173" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L173" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M173" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N173" s="8" t="inlineStr"/>
+      <c r="O173" s="8" t="inlineStr"/>
+      <c r="P173" s="8" t="inlineStr"/>
+      <c r="Q173" s="8" t="inlineStr">
+        <is>
+          <t>Practice state change events</t>
+        </is>
+      </c>
+      <c r="R173" s="8" t="inlineStr">
+        <is>
+          <t>Redis pub/sub practice_status channel</t>
+        </is>
+      </c>
+      <c r="S173" s="8" t="inlineStr"/>
+    </row>
+    <row r="174" ht="30" customHeight="1">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t>proactive_compliance_monitor</t>
+        </is>
+      </c>
+      <c r="B174" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>ogni 24h (86400s)</t>
+        </is>
+      </c>
+      <c r="F174" s="8" t="inlineStr">
+        <is>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+        </is>
+      </c>
+      <c r="G174" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H174" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I174" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J174" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K174" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L174" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M174" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N174" s="8" t="inlineStr"/>
+      <c r="O174" s="8" t="inlineStr"/>
+      <c r="P174" s="8" t="inlineStr"/>
+      <c r="Q174" s="8" t="inlineStr">
+        <is>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
+        </is>
+      </c>
+      <c r="R174" s="8" t="inlineStr">
+        <is>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S174" s="8" t="inlineStr"/>
+    </row>
+    <row r="175" ht="30" customHeight="1">
+      <c r="A175" s="8" t="inlineStr">
+        <is>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F175" s="8" t="inlineStr">
+        <is>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+        </is>
+      </c>
+      <c r="G175" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H175" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I175" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J175" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K175" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L175" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M175" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N175" s="8" t="inlineStr"/>
+      <c r="O175" s="8" t="inlineStr"/>
+      <c r="P175" s="8" t="inlineStr"/>
+      <c r="Q175" s="8" t="inlineStr">
+        <is>
+          <t>Auto-closed timesheet sessions</t>
+        </is>
+      </c>
+      <c r="R175" s="8" t="inlineStr">
+        <is>
+          <t>work_sessions table</t>
+        </is>
+      </c>
+      <c r="S175" s="8" t="inlineStr"/>
+    </row>
+    <row r="176" ht="30" customHeight="1">
+      <c r="A176" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B176" s="17" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C176" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D176" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E176" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F176" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I176" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L176" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M176" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N176" s="8" t="inlineStr"/>
+      <c r="O176" s="8" t="inlineStr"/>
+      <c r="P176" s="8" t="inlineStr"/>
+      <c r="Q176" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R176" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S176" s="8" t="inlineStr"/>
+    </row>
+    <row r="177" ht="30" customHeight="1">
+      <c r="A177" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B177" s="17" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E177" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F177" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G177" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H177" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I177" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J177" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K177" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L177" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M177" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N177" s="8" t="inlineStr"/>
+      <c r="O177" s="8" t="inlineStr"/>
+      <c r="P177" s="8" t="inlineStr"/>
+      <c r="Q177" s="8" t="inlineStr">
+        <is>
+          <t>Twitter match entries</t>
+        </is>
+      </c>
+      <c r="R177" s="8" t="inlineStr">
+        <is>
+          <t>Twitter API v2 search/recent</t>
+        </is>
+      </c>
+      <c r="S177" s="8" t="inlineStr">
+        <is>
+          <t>CRC broken — X API access issues</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>

</xml_diff>

<commit_message>
refactor: merge Intel into Garuda — single intelligence system
Intel (scraping, radar, legal scan) and Garuda (KG consumer, gap
detector) are the same pipeline: Intel is the mouth (collects data),
Garuda is the brain (structures it in Neo4j). Separating them was
a historical artifact, not an architectural decision.

15 automations now under Garuda: intel-pipeline, intel-radar,
normativa-daily, legal_radar, source-enrichment, garuda-consumer,
gap-detector, matagaruda-sentinel/watcher, X monitor, t4-monitor.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/automations-inventory.xlsx
+++ b/docs/automations-inventory.xlsx
@@ -69,7 +69,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -123,11 +123,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -160,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,16 +195,13 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -594,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-14 00:16 WITA</t>
+          <t>Generated: 2026-04-14 00:35 WITA</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1427,7 @@
         </is>
       </c>
       <c r="N6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
@@ -1526,7 +1518,7 @@
         </is>
       </c>
       <c r="N7" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
@@ -2254,7 +2246,7 @@
         </is>
       </c>
       <c r="N15" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
@@ -2531,9 +2523,9 @@
           <t>com.balizero.translate.hourly</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -2662,7 +2654,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L20" s="18" t="inlineStr">
+      <c r="L20" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -2838,7 +2830,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L22" s="18" t="inlineStr">
+      <c r="L22" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -2929,7 +2921,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L23" s="18" t="inlineStr">
+      <c r="L23" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3020,7 +3012,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L24" s="18" t="inlineStr">
+      <c r="L24" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3111,7 +3103,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L25" s="18" t="inlineStr">
+      <c r="L25" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3202,7 +3194,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr">
+      <c r="L26" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3293,7 +3285,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L27" s="18" t="inlineStr">
+      <c r="L27" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3384,7 +3376,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L28" s="18" t="inlineStr">
+      <c r="L28" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -3475,7 +3467,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L29" s="18" t="inlineStr">
+      <c r="L29" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -4010,7 +4002,7 @@
           <t>homebrew.mxcl.postgresql@17</t>
         </is>
       </c>
-      <c r="B36" s="19" t="inlineStr">
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -4334,9 +4326,9 @@
           <t>com.balizero.intel.nightly</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
@@ -4577,7 +4569,7 @@
           <t>com.garuda.consumer.daily</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B43" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -4658,7 +4650,7 @@
           <t>com.garuda.gap-detector.twice-daily</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -4739,7 +4731,7 @@
           <t>com.matagaruda.sentinel.daily</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -4820,7 +4812,7 @@
           <t>com.matagaruda.watcher.daily</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -6282,7 +6274,7 @@
           <t>fly-backup.sh</t>
         </is>
       </c>
-      <c r="B64" s="19" t="inlineStr">
+      <c r="B64" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -6606,9 +6598,9 @@
           <t>intel-scraper-sentinel-bridge.sh</t>
         </is>
       </c>
-      <c r="B68" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B68" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -6687,7 +6679,7 @@
           <t>knowledge-graph-builder.sh</t>
         </is>
       </c>
-      <c r="B69" s="20" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -6768,9 +6760,9 @@
           <t>legal_radar.py</t>
         </is>
       </c>
-      <c r="B70" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -9036,9 +9028,9 @@
           <t>run_overnight.sh</t>
         </is>
       </c>
-      <c r="B98" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
@@ -10050,11 +10042,11 @@
         </is>
       </c>
       <c r="N3" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O3" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:54</t>
+          <t>2026-04-13 16:24</t>
         </is>
       </c>
       <c r="P3" s="8" t="inlineStr">
@@ -10171,9 +10163,9 @@
           <t>nuz-intel-radar</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -10262,9 +10254,9 @@
           <t>nuz-normativa-daily</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -10353,7 +10345,7 @@
           <t>pg-sync-verify</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -10444,9 +10436,9 @@
           <t>source-enrichment-weekly</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -10596,7 +10588,7 @@
         </is>
       </c>
       <c r="N9" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
@@ -10776,9 +10768,9 @@
           <t>intel-pipeline-retry</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -10861,9 +10853,9 @@
           <t>intel-pipeline-scraping</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -11031,7 +11023,7 @@
           <t>pg-sync</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -11509,7 +11501,7 @@
           <t>homebrew.mxcl.postgresql@17</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -13575,7 +13567,7 @@
           <t>fly-pg-backup.sh</t>
         </is>
       </c>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -13899,7 +13891,7 @@
           <t>qdrant-snapshot.sh</t>
         </is>
       </c>
-      <c r="B51" s="19" t="inlineStr">
+      <c r="B51" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -15251,7 +15243,7 @@
           <t>olympus_heartbeat</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -15332,7 +15324,7 @@
           <t>olympus_pulse</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -15656,9 +15648,9 @@
           <t>x_monitor_digest_loop</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -15737,9 +15729,9 @@
           <t>x_monitor_run_loop</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -16380,7 +16372,7 @@
         </is>
       </c>
       <c r="N6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
@@ -16562,11 +16554,11 @@
         </is>
       </c>
       <c r="N8" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>2026-04-13 15:54</t>
+          <t>2026-04-13 16:24</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
@@ -16653,7 +16645,7 @@
         </is>
       </c>
       <c r="N9" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
@@ -16865,9 +16857,9 @@
           <t>nuz-intel-radar</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -16956,9 +16948,9 @@
           <t>nuz-normativa-daily</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -17047,7 +17039,7 @@
           <t>pg-sync-verify</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -17320,9 +17312,9 @@
           <t>source-enrichment-weekly</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -17563,7 +17555,7 @@
         </is>
       </c>
       <c r="N19" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
@@ -17923,7 +17915,7 @@
         </is>
       </c>
       <c r="N23" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O23" s="8" t="inlineStr">
         <is>
@@ -18277,9 +18269,9 @@
           <t>com.balizero.translate.hourly</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -18485,7 +18477,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L30" s="18" t="inlineStr">
+      <c r="L30" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -18526,9 +18518,9 @@
           <t>intel-pipeline-retry</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -18611,9 +18603,9 @@
           <t>intel-pipeline-scraping</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -18831,7 +18823,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L34" s="18" t="inlineStr">
+      <c r="L34" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -18922,7 +18914,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L35" s="18" t="inlineStr">
+      <c r="L35" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19013,7 +19005,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L36" s="18" t="inlineStr">
+      <c r="L36" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19104,7 +19096,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L37" s="18" t="inlineStr">
+      <c r="L37" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19195,7 +19187,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L38" s="18" t="inlineStr">
+      <c r="L38" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19286,7 +19278,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L39" s="18" t="inlineStr">
+      <c r="L39" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19377,7 +19369,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L40" s="18" t="inlineStr">
+      <c r="L40" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19468,7 +19460,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L41" s="18" t="inlineStr">
+      <c r="L41" s="17" t="inlineStr">
         <is>
           <t>skipped</t>
         </is>
@@ -19594,7 +19586,7 @@
           <t>pg-sync</t>
         </is>
       </c>
-      <c r="B43" s="19" t="inlineStr">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -20566,7 +20558,7 @@
           <t>homebrew.mxcl.postgresql@17</t>
         </is>
       </c>
-      <c r="B55" s="19" t="inlineStr">
+      <c r="B55" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -20647,7 +20639,7 @@
           <t>homebrew.mxcl.postgresql@17</t>
         </is>
       </c>
-      <c r="B56" s="19" t="inlineStr">
+      <c r="B56" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -21121,9 +21113,9 @@
           <t>com.balizero.intel.nightly</t>
         </is>
       </c>
-      <c r="B62" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -21364,7 +21356,7 @@
           <t>com.garuda.consumer.daily</t>
         </is>
       </c>
-      <c r="B65" s="20" t="inlineStr">
+      <c r="B65" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -21445,7 +21437,7 @@
           <t>com.garuda.gap-detector.twice-daily</t>
         </is>
       </c>
-      <c r="B66" s="20" t="inlineStr">
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -21526,7 +21518,7 @@
           <t>com.matagaruda.sentinel.daily</t>
         </is>
       </c>
-      <c r="B67" s="20" t="inlineStr">
+      <c r="B67" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -21607,7 +21599,7 @@
           <t>com.matagaruda.watcher.daily</t>
         </is>
       </c>
-      <c r="B68" s="20" t="inlineStr">
+      <c r="B68" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -24904,7 +24896,7 @@
           <t>fly-backup.sh</t>
         </is>
       </c>
-      <c r="B109" s="19" t="inlineStr">
+      <c r="B109" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -25147,7 +25139,7 @@
           <t>fly-pg-backup.sh</t>
         </is>
       </c>
-      <c r="B112" s="19" t="inlineStr">
+      <c r="B112" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -25309,9 +25301,9 @@
           <t>intel-scraper-sentinel-bridge.sh</t>
         </is>
       </c>
-      <c r="B114" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B114" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -25471,7 +25463,7 @@
           <t>knowledge-graph-builder.sh</t>
         </is>
       </c>
-      <c r="B116" s="20" t="inlineStr">
+      <c r="B116" s="19" t="inlineStr">
         <is>
           <t>Garuda</t>
         </is>
@@ -25552,9 +25544,9 @@
           <t>legal_radar.py</t>
         </is>
       </c>
-      <c r="B117" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B117" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
@@ -26119,7 +26111,7 @@
           <t>qdrant-snapshot.sh</t>
         </is>
       </c>
-      <c r="B124" s="19" t="inlineStr">
+      <c r="B124" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -28306,9 +28298,9 @@
           <t>run_overnight.sh</t>
         </is>
       </c>
-      <c r="B151" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B151" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
@@ -29930,7 +29922,7 @@
           <t>olympus_heartbeat</t>
         </is>
       </c>
-      <c r="B171" s="19" t="inlineStr">
+      <c r="B171" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -30011,7 +30003,7 @@
           <t>olympus_pulse</t>
         </is>
       </c>
-      <c r="B172" s="19" t="inlineStr">
+      <c r="B172" s="18" t="inlineStr">
         <is>
           <t>Olympus</t>
         </is>
@@ -30335,9 +30327,9 @@
           <t>x_monitor_digest_loop</t>
         </is>
       </c>
-      <c r="B176" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B176" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C176" s="8" t="inlineStr">
@@ -30416,9 +30408,9 @@
           <t>x_monitor_run_loop</t>
         </is>
       </c>
-      <c r="B177" s="17" t="inlineStr">
-        <is>
-          <t>Intel</t>
+      <c r="B177" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C177" s="8" t="inlineStr">

</xml_diff>

<commit_message>
feat: complete backend services — 18 in-process daemons mapped
Added 7 missing backend workers: Workflow Queue (PG SKIP LOCKED),
Legal Full Ingestion, Attendance Monitor, Daily Checkin Notifier,
Weekly Email Reporter, Notification Scheduler, Channel DLQ Retry.

Total: 183 automations (Pro 105 + Air 60 + Backend 18).
Systems: Ops 56, NLM 40, Sentinel 34, CRM 19, Garuda 16, Olympus 9,
SEO 5, Cell 3.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/automations-inventory.xlsx
+++ b/docs/automations-inventory.xlsx
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-14 00:35 WITA</t>
+          <t>Generated: 2026-04-14 00:39 WITA</t>
         </is>
       </c>
     </row>
@@ -14788,7 +14788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14993,12 +14993,12 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>autonomous_scheduler</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>attendance_monitor</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -15013,12 +15013,12 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (per remaining tasks)</t>
+          <t>escalation periodico + digest 1x/giorno</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
+          <t>Attendance monitor: scans team presence, detects anomalies (late check-in, missed checkout, overtime). Escalation loop + daily digest report.</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
@@ -15061,29 +15061,25 @@
       <c r="P3" s="8" t="inlineStr"/>
       <c r="Q3" s="8" t="inlineStr">
         <is>
-          <t>Self-healing actions</t>
+          <t>Attendance alerts, daily digest</t>
         </is>
       </c>
       <c r="R3" s="8" t="inlineStr">
         <is>
-          <t>Service health status</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
-        </is>
-      </c>
+          <t>work_sessions, team_members tables</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>event_bus_listen</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>autonomous_scheduler</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -15098,12 +15094,12 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven, ping 30s)</t>
+          <t>ogni 5min (per remaining tasks)</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -15146,25 +15142,29 @@
       <c r="P4" s="8" t="inlineStr"/>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>Routed events to subscribers</t>
+          <t>Self-healing actions</t>
         </is>
       </c>
       <c r="R4" s="8" t="inlineStr">
         <is>
-          <t>Redis Streams (all channels)</t>
-        </is>
-      </c>
-      <c r="S4" s="8" t="inlineStr"/>
+          <t>Service health status</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>health_monitor</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>daily_checkin_notifier</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -15179,12 +15179,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>ogni 60s</t>
+          <t>1x/giorno 10:00 WITA</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -15199,7 +15199,7 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Self (top-level monitor)</t>
+          <t>Health Monitor</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -15227,12 +15227,12 @@
       <c r="P5" s="8" t="inlineStr"/>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Service health status, degradation alerts</t>
+          <t>Daily checkin email</t>
         </is>
       </c>
       <c r="R5" s="8" t="inlineStr">
         <is>
-          <t>All internal service health endpoints</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S5" s="8" t="inlineStr"/>
@@ -15240,12 +15240,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>olympus_heartbeat</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>dlq_retry_channels</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -15260,12 +15260,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -15308,12 +15308,12 @@
       <c r="P6" s="8" t="inlineStr"/>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Health metrics, PG stats</t>
+          <t>Retried channel messages</t>
         </is>
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>PostgreSQL pg_stat_statements</t>
+          <t>channel_dlq table</t>
         </is>
       </c>
       <c r="S6" s="8" t="inlineStr"/>
@@ -15321,12 +15321,12 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>olympus_pulse</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -15341,12 +15341,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>continuo (event-driven, ping 30s)</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -15389,12 +15389,12 @@
       <c r="P7" s="8" t="inlineStr"/>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>olympus_insights, PulseAction, alerts</t>
+          <t>Routed events to subscribers</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr">
         <is>
-          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+          <t>Redis Streams (all channels)</t>
         </is>
       </c>
       <c r="S7" s="8" t="inlineStr"/>
@@ -15402,12 +15402,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>practice_status_listener</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -15422,12 +15422,12 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven)</t>
+          <t>ogni 60s</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -15442,7 +15442,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Health Monitor</t>
+          <t>Self (top-level monitor)</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -15470,12 +15470,12 @@
       <c r="P8" s="8" t="inlineStr"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>Practice state change events</t>
+          <t>Service health status, degradation alerts</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
-          <t>Redis pub/sub practice_status channel</t>
+          <t>All internal service health endpoints</t>
         </is>
       </c>
       <c r="S8" s="8" t="inlineStr"/>
@@ -15483,12 +15483,12 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>proactive_compliance_monitor</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>legal_full_ingestion</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -15503,12 +15503,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>ogni 24h (86400s)</t>
+          <t>continuo (poll su coda)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -15551,12 +15551,12 @@
       <c r="P9" s="8" t="inlineStr"/>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Compliance alerts (WhatsApp/Telegram)</t>
+          <t>KB entries (legal documents)</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr">
         <is>
-          <t>CRM practices, client documents</t>
+          <t>legal_ingestion_queue table</t>
         </is>
       </c>
       <c r="S9" s="8" t="inlineStr"/>
@@ -15564,12 +15564,12 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>team_timesheet_auto_logout</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>notification_scheduler</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -15584,12 +15584,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -15632,12 +15632,12 @@
       <c r="P10" s="8" t="inlineStr"/>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Auto-closed timesheet sessions</t>
+          <t>Sent notifications</t>
         </is>
       </c>
       <c r="R10" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>notification_queue table</t>
         </is>
       </c>
       <c r="S10" s="8" t="inlineStr"/>
@@ -15645,12 +15645,12 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_digest_loop</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -15665,12 +15665,12 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>ogni N ore (configurable)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -15713,12 +15713,12 @@
       <c r="P11" s="8" t="inlineStr"/>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Twitter digest report</t>
+          <t>Health metrics, PG stats</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>Stored Twitter matches</t>
+          <t>PostgreSQL pg_stat_statements</t>
         </is>
       </c>
       <c r="S11" s="8" t="inlineStr"/>
@@ -15726,12 +15726,12 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_run_loop</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -15746,12 +15746,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>ogni N minuti (configurable)</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -15794,15 +15794,582 @@
       <c r="P12" s="8" t="inlineStr"/>
       <c r="Q12" s="8" t="inlineStr">
         <is>
+          <t>olympus_insights, PulseAction, alerts</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>practice_status_listener</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr"/>
+      <c r="O13" s="8" t="inlineStr"/>
+      <c r="P13" s="8" t="inlineStr"/>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>Practice state change events</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>Redis pub/sub practice_status channel</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>proactive_compliance_monitor</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>ogni 24h (86400s)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr"/>
+      <c r="O14" s="8" t="inlineStr"/>
+      <c r="P14" s="8" t="inlineStr"/>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr"/>
+      <c r="O15" s="8" t="inlineStr"/>
+      <c r="P15" s="8" t="inlineStr"/>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>Auto-closed timesheet sessions</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>work_sessions table</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>weekly_email_reporter</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Dom 16:00 WITA</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr"/>
+      <c r="O16" s="8" t="inlineStr"/>
+      <c r="P16" s="8" t="inlineStr"/>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>Weekly team email report</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>email_logs, team_members tables</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>workflow_queue</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>continuo (poll su tabella jobs)</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr"/>
+      <c r="O17" s="8" t="inlineStr"/>
+      <c r="P17" s="8" t="inlineStr"/>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Completed workflow results</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr"/>
+      <c r="O18" s="8" t="inlineStr"/>
+      <c r="P18" s="8" t="inlineStr"/>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L19" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr"/>
+      <c r="O19" s="8" t="inlineStr"/>
+      <c r="P19" s="8" t="inlineStr"/>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
           <t>Twitter match entries</t>
         </is>
       </c>
-      <c r="R12" s="8" t="inlineStr">
+      <c r="R19" s="8" t="inlineStr">
         <is>
           <t>Twitter API v2 search/recent</t>
         </is>
       </c>
-      <c r="S12" s="8" t="inlineStr">
+      <c r="S19" s="8" t="inlineStr">
         <is>
           <t>CRC broken — X API access issues</t>
         </is>
@@ -15820,7 +16387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S177"/>
+  <dimension ref="A1:S184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -29672,12 +30239,12 @@
     <row r="168" ht="30" customHeight="1">
       <c r="A168" s="8" t="inlineStr">
         <is>
-          <t>autonomous_scheduler</t>
-        </is>
-      </c>
-      <c r="B168" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>attendance_monitor</t>
+        </is>
+      </c>
+      <c r="B168" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C168" s="8" t="inlineStr">
@@ -29692,12 +30259,12 @@
       </c>
       <c r="E168" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (per remaining tasks)</t>
+          <t>escalation periodico + digest 1x/giorno</t>
         </is>
       </c>
       <c r="F168" s="8" t="inlineStr">
         <is>
-          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
+          <t>Attendance monitor: scans team presence, detects anomalies (late check-in, missed checkout, overtime). Escalation loop + daily digest report.</t>
         </is>
       </c>
       <c r="G168" s="8" t="inlineStr">
@@ -29740,29 +30307,25 @@
       <c r="P168" s="8" t="inlineStr"/>
       <c r="Q168" s="8" t="inlineStr">
         <is>
-          <t>Self-healing actions</t>
+          <t>Attendance alerts, daily digest</t>
         </is>
       </c>
       <c r="R168" s="8" t="inlineStr">
         <is>
-          <t>Service health status</t>
-        </is>
-      </c>
-      <c r="S168" s="8" t="inlineStr">
-        <is>
-          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
-        </is>
-      </c>
+          <t>work_sessions, team_members tables</t>
+        </is>
+      </c>
+      <c r="S168" s="8" t="inlineStr"/>
     </row>
     <row r="169" ht="30" customHeight="1">
       <c r="A169" s="8" t="inlineStr">
         <is>
-          <t>event_bus_listen</t>
-        </is>
-      </c>
-      <c r="B169" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>autonomous_scheduler</t>
+        </is>
+      </c>
+      <c r="B169" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
@@ -29777,12 +30340,12 @@
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven, ping 30s)</t>
+          <t>ogni 5min (per remaining tasks)</t>
         </is>
       </c>
       <c r="F169" s="8" t="inlineStr">
         <is>
-          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+          <t>Backend autonomous scheduler: runs short-interval tasks (&lt;=5min) inside FastAPI process. Long-interval tasks migrated to OpenClaw. Currently: Backend Self-Healing Agent (5min health check).</t>
         </is>
       </c>
       <c r="G169" s="8" t="inlineStr">
@@ -29825,25 +30388,29 @@
       <c r="P169" s="8" t="inlineStr"/>
       <c r="Q169" s="8" t="inlineStr">
         <is>
-          <t>Routed events to subscribers</t>
+          <t>Self-healing actions</t>
         </is>
       </c>
       <c r="R169" s="8" t="inlineStr">
         <is>
-          <t>Redis Streams (all channels)</t>
-        </is>
-      </c>
-      <c r="S169" s="8" t="inlineStr"/>
+          <t>Service health status</t>
+        </is>
+      </c>
+      <c r="S169" s="8" t="inlineStr">
+        <is>
+          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="8" t="inlineStr">
         <is>
-          <t>health_monitor</t>
-        </is>
-      </c>
-      <c r="B170" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>daily_checkin_notifier</t>
+        </is>
+      </c>
+      <c r="B170" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
@@ -29858,12 +30425,12 @@
       </c>
       <c r="E170" s="8" t="inlineStr">
         <is>
-          <t>ogni 60s</t>
+          <t>1x/giorno 10:00 WITA</t>
         </is>
       </c>
       <c r="F170" s="8" t="inlineStr">
         <is>
-          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
         </is>
       </c>
       <c r="G170" s="8" t="inlineStr">
@@ -29878,7 +30445,7 @@
       </c>
       <c r="I170" s="8" t="inlineStr">
         <is>
-          <t>Self (top-level monitor)</t>
+          <t>Health Monitor</t>
         </is>
       </c>
       <c r="J170" s="8" t="inlineStr">
@@ -29906,12 +30473,12 @@
       <c r="P170" s="8" t="inlineStr"/>
       <c r="Q170" s="8" t="inlineStr">
         <is>
-          <t>Service health status, degradation alerts</t>
+          <t>Daily checkin email</t>
         </is>
       </c>
       <c r="R170" s="8" t="inlineStr">
         <is>
-          <t>All internal service health endpoints</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -29919,12 +30486,12 @@
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="8" t="inlineStr">
         <is>
-          <t>olympus_heartbeat</t>
-        </is>
-      </c>
-      <c r="B171" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>dlq_retry_channels</t>
+        </is>
+      </c>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C171" s="8" t="inlineStr">
@@ -29939,12 +30506,12 @@
       </c>
       <c r="E171" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F171" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
         </is>
       </c>
       <c r="G171" s="8" t="inlineStr">
@@ -29987,12 +30554,12 @@
       <c r="P171" s="8" t="inlineStr"/>
       <c r="Q171" s="8" t="inlineStr">
         <is>
-          <t>Health metrics, PG stats</t>
+          <t>Retried channel messages</t>
         </is>
       </c>
       <c r="R171" s="8" t="inlineStr">
         <is>
-          <t>PostgreSQL pg_stat_statements</t>
+          <t>channel_dlq table</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -30000,12 +30567,12 @@
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="8" t="inlineStr">
         <is>
-          <t>olympus_pulse</t>
-        </is>
-      </c>
-      <c r="B172" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B172" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C172" s="8" t="inlineStr">
@@ -30020,12 +30587,12 @@
       </c>
       <c r="E172" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>continuo (event-driven, ping 30s)</t>
         </is>
       </c>
       <c r="F172" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
         </is>
       </c>
       <c r="G172" s="8" t="inlineStr">
@@ -30068,12 +30635,12 @@
       <c r="P172" s="8" t="inlineStr"/>
       <c r="Q172" s="8" t="inlineStr">
         <is>
-          <t>olympus_insights, PulseAction, alerts</t>
+          <t>Routed events to subscribers</t>
         </is>
       </c>
       <c r="R172" s="8" t="inlineStr">
         <is>
-          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+          <t>Redis Streams (all channels)</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -30081,12 +30648,12 @@
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="8" t="inlineStr">
         <is>
-          <t>practice_status_listener</t>
-        </is>
-      </c>
-      <c r="B173" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B173" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C173" s="8" t="inlineStr">
@@ -30101,12 +30668,12 @@
       </c>
       <c r="E173" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven)</t>
+          <t>ogni 60s</t>
         </is>
       </c>
       <c r="F173" s="8" t="inlineStr">
         <is>
-          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
         </is>
       </c>
       <c r="G173" s="8" t="inlineStr">
@@ -30121,7 +30688,7 @@
       </c>
       <c r="I173" s="8" t="inlineStr">
         <is>
-          <t>Health Monitor</t>
+          <t>Self (top-level monitor)</t>
         </is>
       </c>
       <c r="J173" s="8" t="inlineStr">
@@ -30149,12 +30716,12 @@
       <c r="P173" s="8" t="inlineStr"/>
       <c r="Q173" s="8" t="inlineStr">
         <is>
-          <t>Practice state change events</t>
+          <t>Service health status, degradation alerts</t>
         </is>
       </c>
       <c r="R173" s="8" t="inlineStr">
         <is>
-          <t>Redis pub/sub practice_status channel</t>
+          <t>All internal service health endpoints</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -30162,12 +30729,12 @@
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="8" t="inlineStr">
         <is>
-          <t>proactive_compliance_monitor</t>
-        </is>
-      </c>
-      <c r="B174" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>legal_full_ingestion</t>
+        </is>
+      </c>
+      <c r="B174" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C174" s="8" t="inlineStr">
@@ -30182,12 +30749,12 @@
       </c>
       <c r="E174" s="8" t="inlineStr">
         <is>
-          <t>ogni 24h (86400s)</t>
+          <t>continuo (poll su coda)</t>
         </is>
       </c>
       <c r="F174" s="8" t="inlineStr">
         <is>
-          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
         </is>
       </c>
       <c r="G174" s="8" t="inlineStr">
@@ -30230,12 +30797,12 @@
       <c r="P174" s="8" t="inlineStr"/>
       <c r="Q174" s="8" t="inlineStr">
         <is>
-          <t>Compliance alerts (WhatsApp/Telegram)</t>
+          <t>KB entries (legal documents)</t>
         </is>
       </c>
       <c r="R174" s="8" t="inlineStr">
         <is>
-          <t>CRM practices, client documents</t>
+          <t>legal_ingestion_queue table</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -30243,12 +30810,12 @@
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="8" t="inlineStr">
         <is>
-          <t>team_timesheet_auto_logout</t>
-        </is>
-      </c>
-      <c r="B175" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>notification_scheduler</t>
+        </is>
+      </c>
+      <c r="B175" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C175" s="8" t="inlineStr">
@@ -30263,12 +30830,12 @@
       </c>
       <c r="E175" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
         </is>
       </c>
       <c r="G175" s="8" t="inlineStr">
@@ -30311,12 +30878,12 @@
       <c r="P175" s="8" t="inlineStr"/>
       <c r="Q175" s="8" t="inlineStr">
         <is>
-          <t>Auto-closed timesheet sessions</t>
+          <t>Sent notifications</t>
         </is>
       </c>
       <c r="R175" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>notification_queue table</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -30324,12 +30891,12 @@
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_digest_loop</t>
-        </is>
-      </c>
-      <c r="B176" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B176" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C176" s="8" t="inlineStr">
@@ -30344,12 +30911,12 @@
       </c>
       <c r="E176" s="8" t="inlineStr">
         <is>
-          <t>ogni N ore (configurable)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F176" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
         </is>
       </c>
       <c r="G176" s="8" t="inlineStr">
@@ -30392,12 +30959,12 @@
       <c r="P176" s="8" t="inlineStr"/>
       <c r="Q176" s="8" t="inlineStr">
         <is>
-          <t>Twitter digest report</t>
+          <t>Health metrics, PG stats</t>
         </is>
       </c>
       <c r="R176" s="8" t="inlineStr">
         <is>
-          <t>Stored Twitter matches</t>
+          <t>PostgreSQL pg_stat_statements</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -30405,12 +30972,12 @@
     <row r="177" ht="30" customHeight="1">
       <c r="A177" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_run_loop</t>
-        </is>
-      </c>
-      <c r="B177" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B177" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C177" s="8" t="inlineStr">
@@ -30425,12 +30992,12 @@
       </c>
       <c r="E177" s="8" t="inlineStr">
         <is>
-          <t>ogni N minuti (configurable)</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="F177" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
         </is>
       </c>
       <c r="G177" s="8" t="inlineStr">
@@ -30473,15 +31040,582 @@
       <c r="P177" s="8" t="inlineStr"/>
       <c r="Q177" s="8" t="inlineStr">
         <is>
+          <t>olympus_insights, PulseAction, alerts</t>
+        </is>
+      </c>
+      <c r="R177" s="8" t="inlineStr">
+        <is>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+        </is>
+      </c>
+      <c r="S177" s="8" t="inlineStr"/>
+    </row>
+    <row r="178" ht="30" customHeight="1">
+      <c r="A178" s="8" t="inlineStr">
+        <is>
+          <t>practice_status_listener</t>
+        </is>
+      </c>
+      <c r="B178" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C178" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D178" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E178" s="8" t="inlineStr">
+        <is>
+          <t>continuo (event-driven)</t>
+        </is>
+      </c>
+      <c r="F178" s="8" t="inlineStr">
+        <is>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+        </is>
+      </c>
+      <c r="G178" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H178" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I178" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J178" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K178" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L178" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M178" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N178" s="8" t="inlineStr"/>
+      <c r="O178" s="8" t="inlineStr"/>
+      <c r="P178" s="8" t="inlineStr"/>
+      <c r="Q178" s="8" t="inlineStr">
+        <is>
+          <t>Practice state change events</t>
+        </is>
+      </c>
+      <c r="R178" s="8" t="inlineStr">
+        <is>
+          <t>Redis pub/sub practice_status channel</t>
+        </is>
+      </c>
+      <c r="S178" s="8" t="inlineStr"/>
+    </row>
+    <row r="179" ht="30" customHeight="1">
+      <c r="A179" s="8" t="inlineStr">
+        <is>
+          <t>proactive_compliance_monitor</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C179" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E179" s="8" t="inlineStr">
+        <is>
+          <t>ogni 24h (86400s)</t>
+        </is>
+      </c>
+      <c r="F179" s="8" t="inlineStr">
+        <is>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+        </is>
+      </c>
+      <c r="G179" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H179" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I179" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J179" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K179" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L179" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M179" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N179" s="8" t="inlineStr"/>
+      <c r="O179" s="8" t="inlineStr"/>
+      <c r="P179" s="8" t="inlineStr"/>
+      <c r="Q179" s="8" t="inlineStr">
+        <is>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
+        </is>
+      </c>
+      <c r="R179" s="8" t="inlineStr">
+        <is>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S179" s="8" t="inlineStr"/>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="8" t="inlineStr">
+        <is>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B180" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C180" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D180" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E180" s="8" t="inlineStr">
+        <is>
+          <t>ogni 5min (300s)</t>
+        </is>
+      </c>
+      <c r="F180" s="8" t="inlineStr">
+        <is>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+        </is>
+      </c>
+      <c r="G180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I180" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L180" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M180" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N180" s="8" t="inlineStr"/>
+      <c r="O180" s="8" t="inlineStr"/>
+      <c r="P180" s="8" t="inlineStr"/>
+      <c r="Q180" s="8" t="inlineStr">
+        <is>
+          <t>Auto-closed timesheet sessions</t>
+        </is>
+      </c>
+      <c r="R180" s="8" t="inlineStr">
+        <is>
+          <t>work_sessions table</t>
+        </is>
+      </c>
+      <c r="S180" s="8" t="inlineStr"/>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="8" t="inlineStr">
+        <is>
+          <t>weekly_email_reporter</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C181" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E181" s="8" t="inlineStr">
+        <is>
+          <t>Dom 16:00 WITA</t>
+        </is>
+      </c>
+      <c r="F181" s="8" t="inlineStr">
+        <is>
+          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
+        </is>
+      </c>
+      <c r="G181" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H181" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I181" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J181" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K181" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L181" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M181" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N181" s="8" t="inlineStr"/>
+      <c r="O181" s="8" t="inlineStr"/>
+      <c r="P181" s="8" t="inlineStr"/>
+      <c r="Q181" s="8" t="inlineStr">
+        <is>
+          <t>Weekly team email report</t>
+        </is>
+      </c>
+      <c r="R181" s="8" t="inlineStr">
+        <is>
+          <t>email_logs, team_members tables</t>
+        </is>
+      </c>
+      <c r="S181" s="8" t="inlineStr"/>
+    </row>
+    <row r="182" ht="30" customHeight="1">
+      <c r="A182" s="8" t="inlineStr">
+        <is>
+          <t>workflow_queue</t>
+        </is>
+      </c>
+      <c r="B182" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C182" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D182" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E182" s="8" t="inlineStr">
+        <is>
+          <t>continuo (poll su tabella jobs)</t>
+        </is>
+      </c>
+      <c r="F182" s="8" t="inlineStr">
+        <is>
+          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+        </is>
+      </c>
+      <c r="G182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I182" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L182" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M182" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N182" s="8" t="inlineStr"/>
+      <c r="O182" s="8" t="inlineStr"/>
+      <c r="P182" s="8" t="inlineStr"/>
+      <c r="Q182" s="8" t="inlineStr">
+        <is>
+          <t>Completed workflow results</t>
+        </is>
+      </c>
+      <c r="R182" s="8" t="inlineStr">
+        <is>
+          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+        </is>
+      </c>
+      <c r="S182" s="8" t="inlineStr"/>
+    </row>
+    <row r="183" ht="30" customHeight="1">
+      <c r="A183" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B183" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C183" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E183" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G183" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H183" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I183" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J183" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K183" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L183" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M183" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N183" s="8" t="inlineStr"/>
+      <c r="O183" s="8" t="inlineStr"/>
+      <c r="P183" s="8" t="inlineStr"/>
+      <c r="Q183" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R183" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S183" s="8" t="inlineStr"/>
+    </row>
+    <row r="184" ht="30" customHeight="1">
+      <c r="A184" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B184" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C184" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D184" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E184" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F184" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I184" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L184" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M184" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N184" s="8" t="inlineStr"/>
+      <c r="O184" s="8" t="inlineStr"/>
+      <c r="P184" s="8" t="inlineStr"/>
+      <c r="Q184" s="8" t="inlineStr">
+        <is>
           <t>Twitter match entries</t>
         </is>
       </c>
-      <c r="R177" s="8" t="inlineStr">
+      <c r="R184" s="8" t="inlineStr">
         <is>
           <t>Twitter API v2 search/recent</t>
         </is>
       </c>
-      <c r="S177" s="8" t="inlineStr">
+      <c r="S184" s="8" t="inlineStr">
         <is>
           <t>CRC broken — X API access issues</t>
         </is>

</xml_diff>

<commit_message>
fix: audit findings from 4 agents — 186 automations verified
Added 3 backend services, 5 zombie entries, fixed 11 schedules,
marked 4 disabled services.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/automations-inventory.xlsx
+++ b/docs/automations-inventory.xlsx
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-14 00:39 WITA</t>
+          <t>Generated: 2026-04-14 00:55 WITA</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="N6" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>ogni ora :30</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>09:00 WITA</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>01:00 WITA (nightly)</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>08:00 WITA</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>06:15 WITA</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>07:00 + 18:00 WITA</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>02:00 WITA</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>06:00 WITA</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>23:15 WITA</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>10:00 WITA</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -5724,7 +5724,7 @@
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>Lun 09:00 WITA</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -14788,7 +14788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14988,7 +14988,11 @@
           <t>Individual alert events</t>
         </is>
       </c>
-      <c r="S2" s="8" t="inlineStr"/>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>Runs via legacy startup.py:43, not service_initializer.py. Verify if startup.py is still in the boot path.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
@@ -15152,19 +15156,19 @@
       </c>
       <c r="S4" s="8" t="inlineStr">
         <is>
-          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+          <t>DISABLED — _init_background_services() commented out in service_initializer.py:1169. Only HealthMonitor runs.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>daily_checkin_notifier</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>confirmation_pubsub_listener</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -15179,12 +15183,12 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>1x/giorno 10:00 WITA</t>
+          <t>continuo (Redis pub/sub)</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
+          <t>Confirmation service pub/sub listener: persistent Redis subscriber on conf:resolutions channel. Resolves async confirmation Futures when agent confirmations arrive.</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -15227,12 +15231,12 @@
       <c r="P5" s="8" t="inlineStr"/>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Daily checkin email</t>
+          <t>Resolved confirmation Futures</t>
         </is>
       </c>
       <c r="R5" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>Redis channel conf:resolutions</t>
         </is>
       </c>
       <c r="S5" s="8" t="inlineStr"/>
@@ -15240,12 +15244,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>dlq_retry_channels</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>daily_checkin_notifier</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -15260,12 +15264,12 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>continuo</t>
+          <t>1x/giorno 10:00 WITA</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
+          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -15308,12 +15312,12 @@
       <c r="P6" s="8" t="inlineStr"/>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Retried channel messages</t>
+          <t>Daily checkin email</t>
         </is>
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>channel_dlq table</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S6" s="8" t="inlineStr"/>
@@ -15321,12 +15325,12 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>event_bus_listen</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>database_health_check_loop</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -15341,12 +15345,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven, ping 30s)</t>
+          <t>ogni 15s</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+          <t>Database health check: verifies asyncpg pool is healthy every 15s. Detects stale connections, pool exhaustion, InterfaceError recovery.</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -15389,12 +15393,12 @@
       <c r="P7" s="8" t="inlineStr"/>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Routed events to subscribers</t>
+          <t>DB pool health status, auto-reconnect</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr">
         <is>
-          <t>Redis Streams (all channels)</t>
+          <t>asyncpg pool stats</t>
         </is>
       </c>
       <c r="S7" s="8" t="inlineStr"/>
@@ -15402,12 +15406,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>health_monitor</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>dlq_retry_channels</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -15422,12 +15426,12 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>ogni 60s</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -15442,7 +15446,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Self (top-level monitor)</t>
+          <t>Health Monitor</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -15470,12 +15474,12 @@
       <c r="P8" s="8" t="inlineStr"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>Service health status, degradation alerts</t>
+          <t>Retried channel messages</t>
         </is>
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
-          <t>All internal service health endpoints</t>
+          <t>channel_dlq table</t>
         </is>
       </c>
       <c r="S8" s="8" t="inlineStr"/>
@@ -15483,12 +15487,12 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>legal_full_ingestion</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -15503,12 +15507,12 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>continuo (poll su coda)</t>
+          <t>continuo (event-driven, ping 30s)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -15551,12 +15555,12 @@
       <c r="P9" s="8" t="inlineStr"/>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>KB entries (legal documents)</t>
+          <t>Routed events to subscribers</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr">
         <is>
-          <t>legal_ingestion_queue table</t>
+          <t>Redis Streams (all channels)</t>
         </is>
       </c>
       <c r="S9" s="8" t="inlineStr"/>
@@ -15564,12 +15568,12 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>notification_scheduler</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -15584,12 +15588,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>continuo</t>
+          <t>ogni 60s</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -15604,7 +15608,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Health Monitor</t>
+          <t>Self (top-level monitor)</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -15632,12 +15636,12 @@
       <c r="P10" s="8" t="inlineStr"/>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Sent notifications</t>
+          <t>Service health status, degradation alerts</t>
         </is>
       </c>
       <c r="R10" s="8" t="inlineStr">
         <is>
-          <t>notification_queue table</t>
+          <t>All internal service health endpoints</t>
         </is>
       </c>
       <c r="S10" s="8" t="inlineStr"/>
@@ -15645,12 +15649,12 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>olympus_heartbeat</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>legal_full_ingestion</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -15665,12 +15669,12 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo (poll su coda)</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -15713,12 +15717,12 @@
       <c r="P11" s="8" t="inlineStr"/>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Health metrics, PG stats</t>
+          <t>KB entries (legal documents)</t>
         </is>
       </c>
       <c r="R11" s="8" t="inlineStr">
         <is>
-          <t>PostgreSQL pg_stat_statements</t>
+          <t>legal_ingestion_queue table</t>
         </is>
       </c>
       <c r="S11" s="8" t="inlineStr"/>
@@ -15726,12 +15730,12 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>olympus_pulse</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>notification_scheduler</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -15746,12 +15750,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -15794,12 +15798,12 @@
       <c r="P12" s="8" t="inlineStr"/>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>olympus_insights, PulseAction, alerts</t>
+          <t>Sent notifications</t>
         </is>
       </c>
       <c r="R12" s="8" t="inlineStr">
         <is>
-          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+          <t>notification_queue table</t>
         </is>
       </c>
       <c r="S12" s="8" t="inlineStr"/>
@@ -15807,12 +15811,12 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>practice_status_listener</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -15827,12 +15831,12 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -15875,12 +15879,12 @@
       <c r="P13" s="8" t="inlineStr"/>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>Practice state change events</t>
+          <t>Health metrics, PG stats</t>
         </is>
       </c>
       <c r="R13" s="8" t="inlineStr">
         <is>
-          <t>Redis pub/sub practice_status channel</t>
+          <t>PostgreSQL pg_stat_statements</t>
         </is>
       </c>
       <c r="S13" s="8" t="inlineStr"/>
@@ -15888,12 +15892,12 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>proactive_compliance_monitor</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -15908,12 +15912,12 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>ogni 24h (86400s)</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -15956,12 +15960,12 @@
       <c r="P14" s="8" t="inlineStr"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>Compliance alerts (WhatsApp/Telegram)</t>
+          <t>olympus_insights, PulseAction, alerts</t>
         </is>
       </c>
       <c r="R14" s="8" t="inlineStr">
         <is>
-          <t>CRM practices, client documents</t>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
         </is>
       </c>
       <c r="S14" s="8" t="inlineStr"/>
@@ -15969,7 +15973,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>team_timesheet_auto_logout</t>
+          <t>practice_status_listener</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -15989,12 +15993,12 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo (event-driven)</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -16037,12 +16041,12 @@
       <c r="P15" s="8" t="inlineStr"/>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>Auto-closed timesheet sessions</t>
+          <t>Practice state change events</t>
         </is>
       </c>
       <c r="R15" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>Redis pub/sub practice_status channel</t>
         </is>
       </c>
       <c r="S15" s="8" t="inlineStr"/>
@@ -16050,7 +16054,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>weekly_email_reporter</t>
+          <t>proactive_compliance_monitor</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -16070,12 +16074,12 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Dom 16:00 WITA</t>
+          <t>ogni 24h (86400s)</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -16118,25 +16122,29 @@
       <c r="P16" s="8" t="inlineStr"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>Weekly team email report</t>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
         </is>
       </c>
       <c r="R16" s="8" t="inlineStr">
         <is>
-          <t>email_logs, team_members tables</t>
-        </is>
-      </c>
-      <c r="S16" s="8" t="inlineStr"/>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — _init_background_services() commented out. Re-enable when omnichannel stabilization complete.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>workflow_queue</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -16151,12 +16159,12 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>continuo (poll su tabella jobs)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -16199,12 +16207,12 @@
       <c r="P17" s="8" t="inlineStr"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Completed workflow results</t>
+          <t>Auto-closed timesheet sessions</t>
         </is>
       </c>
       <c r="R17" s="8" t="inlineStr">
         <is>
-          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S17" s="8" t="inlineStr"/>
@@ -16212,12 +16220,12 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_digest_loop</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>websocket_redis_listener</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -16232,12 +16240,12 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>ogni N ore (configurable)</t>
+          <t>continuo (Redis→WebSocket bridge)</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+          <t>WebSocket Redis bridge: persistent background task that relays Redis pub/sub messages to connected WebSocket clients for real-time UI updates.</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
@@ -16280,12 +16288,12 @@
       <c r="P18" s="8" t="inlineStr"/>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Twitter digest report</t>
+          <t>Real-time WebSocket messages to frontend</t>
         </is>
       </c>
       <c r="R18" s="8" t="inlineStr">
         <is>
-          <t>Stored Twitter matches</t>
+          <t>Redis pub/sub channels</t>
         </is>
       </c>
       <c r="S18" s="8" t="inlineStr"/>
@@ -16293,12 +16301,12 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_run_loop</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>weekly_email_reporter</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -16313,12 +16321,12 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>ogni N minuti (configurable)</t>
+          <t>Dom 16:00 WITA</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -16361,17 +16369,264 @@
       <c r="P19" s="8" t="inlineStr"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
+          <t>Weekly team email report</t>
+        </is>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t>email_logs, team_members tables</t>
+        </is>
+      </c>
+      <c r="S19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>workflow_queue</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>continuo (poll su tabella jobs)</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L20" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr"/>
+      <c r="O20" s="8" t="inlineStr"/>
+      <c r="P20" s="8" t="inlineStr"/>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>Completed workflow results</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+        </is>
+      </c>
+      <c r="S20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L21" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr"/>
+      <c r="O21" s="8" t="inlineStr"/>
+      <c r="P21" s="8" t="inlineStr"/>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S21" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — same as x_monitor_run_loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr"/>
+      <c r="O22" s="8" t="inlineStr"/>
+      <c r="P22" s="8" t="inlineStr"/>
+      <c r="Q22" s="8" t="inlineStr">
+        <is>
           <t>Twitter match entries</t>
         </is>
       </c>
-      <c r="R19" s="8" t="inlineStr">
+      <c r="R22" s="8" t="inlineStr">
         <is>
           <t>Twitter API v2 search/recent</t>
         </is>
       </c>
-      <c r="S19" s="8" t="inlineStr">
-        <is>
-          <t>CRC broken — X API access issues</t>
+      <c r="S22" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — loops exist in code but no startup wiring in service_initializer.py. X/Twitter CRC also broken.</t>
         </is>
       </c>
     </row>
@@ -16387,7 +16642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S184"/>
+  <dimension ref="A1:S187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16939,7 +17194,7 @@
         </is>
       </c>
       <c r="N6" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
@@ -18853,7 +19108,7 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>ogni ora :30</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -21616,7 +21871,7 @@
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>09:00 WITA</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -21697,7 +21952,7 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>01:00 WITA (nightly)</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -21859,7 +22114,7 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>08:00 WITA</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -21940,7 +22195,7 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>06:15 WITA</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -22021,7 +22276,7 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>07:00 + 18:00 WITA</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -22102,7 +22357,7 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>02:00 WITA</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -22183,7 +22438,7 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>06:00 WITA</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -22345,7 +22600,7 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>23:15 WITA</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -23374,7 +23629,7 @@
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>10:00 WITA</t>
         </is>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -23540,7 +23795,7 @@
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>at boot</t>
+          <t>Lun 09:00 WITA</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
@@ -30234,7 +30489,11 @@
           <t>Individual alert events</t>
         </is>
       </c>
-      <c r="S167" s="8" t="inlineStr"/>
+      <c r="S167" s="8" t="inlineStr">
+        <is>
+          <t>Runs via legacy startup.py:43, not service_initializer.py. Verify if startup.py is still in the boot path.</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="30" customHeight="1">
       <c r="A168" s="8" t="inlineStr">
@@ -30398,19 +30657,19 @@
       </c>
       <c r="S169" s="8" t="inlineStr">
         <is>
-          <t>Most tasks migrated to OpenClaw cron. Only short-interval tasks remain.</t>
+          <t>DISABLED — _init_background_services() commented out in service_initializer.py:1169. Only HealthMonitor runs.</t>
         </is>
       </c>
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="8" t="inlineStr">
         <is>
-          <t>daily_checkin_notifier</t>
-        </is>
-      </c>
-      <c r="B170" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>confirmation_pubsub_listener</t>
+        </is>
+      </c>
+      <c r="B170" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
@@ -30425,12 +30684,12 @@
       </c>
       <c r="E170" s="8" t="inlineStr">
         <is>
-          <t>1x/giorno 10:00 WITA</t>
+          <t>continuo (Redis pub/sub)</t>
         </is>
       </c>
       <c r="F170" s="8" t="inlineStr">
         <is>
-          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
+          <t>Confirmation service pub/sub listener: persistent Redis subscriber on conf:resolutions channel. Resolves async confirmation Futures when agent confirmations arrive.</t>
         </is>
       </c>
       <c r="G170" s="8" t="inlineStr">
@@ -30473,12 +30732,12 @@
       <c r="P170" s="8" t="inlineStr"/>
       <c r="Q170" s="8" t="inlineStr">
         <is>
-          <t>Daily checkin email</t>
+          <t>Resolved confirmation Futures</t>
         </is>
       </c>
       <c r="R170" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>Redis channel conf:resolutions</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -30486,12 +30745,12 @@
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="8" t="inlineStr">
         <is>
-          <t>dlq_retry_channels</t>
-        </is>
-      </c>
-      <c r="B171" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>daily_checkin_notifier</t>
+        </is>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C171" s="8" t="inlineStr">
@@ -30506,12 +30765,12 @@
       </c>
       <c r="E171" s="8" t="inlineStr">
         <is>
-          <t>continuo</t>
+          <t>1x/giorno 10:00 WITA</t>
         </is>
       </c>
       <c r="F171" s="8" t="inlineStr">
         <is>
-          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
+          <t>Daily checkin email: sends morning email to zero@balizero.com with team check-in status summary.</t>
         </is>
       </c>
       <c r="G171" s="8" t="inlineStr">
@@ -30554,12 +30813,12 @@
       <c r="P171" s="8" t="inlineStr"/>
       <c r="Q171" s="8" t="inlineStr">
         <is>
-          <t>Retried channel messages</t>
+          <t>Daily checkin email</t>
         </is>
       </c>
       <c r="R171" s="8" t="inlineStr">
         <is>
-          <t>channel_dlq table</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -30567,12 +30826,12 @@
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="8" t="inlineStr">
         <is>
-          <t>event_bus_listen</t>
-        </is>
-      </c>
-      <c r="B172" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>database_health_check_loop</t>
+        </is>
+      </c>
+      <c r="B172" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C172" s="8" t="inlineStr">
@@ -30587,12 +30846,12 @@
       </c>
       <c r="E172" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven, ping 30s)</t>
+          <t>ogni 15s</t>
         </is>
       </c>
       <c r="F172" s="8" t="inlineStr">
         <is>
-          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
+          <t>Database health check: verifies asyncpg pool is healthy every 15s. Detects stale connections, pool exhaustion, InterfaceError recovery.</t>
         </is>
       </c>
       <c r="G172" s="8" t="inlineStr">
@@ -30635,12 +30894,12 @@
       <c r="P172" s="8" t="inlineStr"/>
       <c r="Q172" s="8" t="inlineStr">
         <is>
-          <t>Routed events to subscribers</t>
+          <t>DB pool health status, auto-reconnect</t>
         </is>
       </c>
       <c r="R172" s="8" t="inlineStr">
         <is>
-          <t>Redis Streams (all channels)</t>
+          <t>asyncpg pool stats</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -30648,12 +30907,12 @@
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="8" t="inlineStr">
         <is>
-          <t>health_monitor</t>
-        </is>
-      </c>
-      <c r="B173" s="12" t="inlineStr">
-        <is>
-          <t>Sentinel</t>
+          <t>dlq_retry_channels</t>
+        </is>
+      </c>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C173" s="8" t="inlineStr">
@@ -30668,12 +30927,12 @@
       </c>
       <c r="E173" s="8" t="inlineStr">
         <is>
-          <t>ogni 60s</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F173" s="8" t="inlineStr">
         <is>
-          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
+          <t>Channel DLQ retry: dead letter queue for failed channel messages (WhatsApp/Telegram/Instagram). Automatic retry with exponential backoff.</t>
         </is>
       </c>
       <c r="G173" s="8" t="inlineStr">
@@ -30688,7 +30947,7 @@
       </c>
       <c r="I173" s="8" t="inlineStr">
         <is>
-          <t>Self (top-level monitor)</t>
+          <t>Health Monitor</t>
         </is>
       </c>
       <c r="J173" s="8" t="inlineStr">
@@ -30716,12 +30975,12 @@
       <c r="P173" s="8" t="inlineStr"/>
       <c r="Q173" s="8" t="inlineStr">
         <is>
-          <t>Service health status, degradation alerts</t>
+          <t>Retried channel messages</t>
         </is>
       </c>
       <c r="R173" s="8" t="inlineStr">
         <is>
-          <t>All internal service health endpoints</t>
+          <t>channel_dlq table</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -30729,12 +30988,12 @@
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="8" t="inlineStr">
         <is>
-          <t>legal_full_ingestion</t>
-        </is>
-      </c>
-      <c r="B174" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>event_bus_listen</t>
+        </is>
+      </c>
+      <c r="B174" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C174" s="8" t="inlineStr">
@@ -30749,12 +31008,12 @@
       </c>
       <c r="E174" s="8" t="inlineStr">
         <is>
-          <t>continuo (poll su coda)</t>
+          <t>continuo (event-driven, ping 30s)</t>
         </is>
       </c>
       <c r="F174" s="8" t="inlineStr">
         <is>
-          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
+          <t>EventBus listener: Redis Streams consumer for inter-service communication. Routes events between services. Core nervous system.</t>
         </is>
       </c>
       <c r="G174" s="8" t="inlineStr">
@@ -30797,12 +31056,12 @@
       <c r="P174" s="8" t="inlineStr"/>
       <c r="Q174" s="8" t="inlineStr">
         <is>
-          <t>KB entries (legal documents)</t>
+          <t>Routed events to subscribers</t>
         </is>
       </c>
       <c r="R174" s="8" t="inlineStr">
         <is>
-          <t>legal_ingestion_queue table</t>
+          <t>Redis Streams (all channels)</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -30810,12 +31069,12 @@
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="8" t="inlineStr">
         <is>
-          <t>notification_scheduler</t>
-        </is>
-      </c>
-      <c r="B175" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>health_monitor</t>
+        </is>
+      </c>
+      <c r="B175" s="12" t="inlineStr">
+        <is>
+          <t>Sentinel</t>
         </is>
       </c>
       <c r="C175" s="8" t="inlineStr">
@@ -30830,12 +31089,12 @@
       </c>
       <c r="E175" s="8" t="inlineStr">
         <is>
-          <t>continuo</t>
+          <t>ogni 60s</t>
         </is>
       </c>
       <c r="F175" s="8" t="inlineStr">
         <is>
-          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
+          <t>Backend health monitor: checks all internal services (DB, Redis, Qdrant, Ollama tunnel, EventBus) every 60s. Core observability.</t>
         </is>
       </c>
       <c r="G175" s="8" t="inlineStr">
@@ -30850,7 +31109,7 @@
       </c>
       <c r="I175" s="8" t="inlineStr">
         <is>
-          <t>Health Monitor</t>
+          <t>Self (top-level monitor)</t>
         </is>
       </c>
       <c r="J175" s="8" t="inlineStr">
@@ -30878,12 +31137,12 @@
       <c r="P175" s="8" t="inlineStr"/>
       <c r="Q175" s="8" t="inlineStr">
         <is>
-          <t>Sent notifications</t>
+          <t>Service health status, degradation alerts</t>
         </is>
       </c>
       <c r="R175" s="8" t="inlineStr">
         <is>
-          <t>notification_queue table</t>
+          <t>All internal service health endpoints</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -30891,12 +31150,12 @@
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="8" t="inlineStr">
         <is>
-          <t>olympus_heartbeat</t>
-        </is>
-      </c>
-      <c r="B176" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>legal_full_ingestion</t>
+        </is>
+      </c>
+      <c r="B176" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
         </is>
       </c>
       <c r="C176" s="8" t="inlineStr">
@@ -30911,12 +31170,12 @@
       </c>
       <c r="E176" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo (poll su coda)</t>
         </is>
       </c>
       <c r="F176" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
+          <t>Legal document ingestion: background processing of legal documents via PG SKIP LOCKED queue. Parses, extracts, indexes into KB.</t>
         </is>
       </c>
       <c r="G176" s="8" t="inlineStr">
@@ -30959,12 +31218,12 @@
       <c r="P176" s="8" t="inlineStr"/>
       <c r="Q176" s="8" t="inlineStr">
         <is>
-          <t>Health metrics, PG stats</t>
+          <t>KB entries (legal documents)</t>
         </is>
       </c>
       <c r="R176" s="8" t="inlineStr">
         <is>
-          <t>PostgreSQL pg_stat_statements</t>
+          <t>legal_ingestion_queue table</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -30972,12 +31231,12 @@
     <row r="177" ht="30" customHeight="1">
       <c r="A177" s="8" t="inlineStr">
         <is>
-          <t>olympus_pulse</t>
-        </is>
-      </c>
-      <c r="B177" s="18" t="inlineStr">
-        <is>
-          <t>Olympus</t>
+          <t>notification_scheduler</t>
+        </is>
+      </c>
+      <c r="B177" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C177" s="8" t="inlineStr">
@@ -30992,12 +31251,12 @@
       </c>
       <c r="E177" s="8" t="inlineStr">
         <is>
-          <t>ogni 6h</t>
+          <t>continuo</t>
         </is>
       </c>
       <c r="F177" s="8" t="inlineStr">
         <is>
-          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
+          <t>Notification scheduler: generic notification dispatch engine. Processes queued notifications (email, WhatsApp, Telegram) with rate limiting.</t>
         </is>
       </c>
       <c r="G177" s="8" t="inlineStr">
@@ -31040,12 +31299,12 @@
       <c r="P177" s="8" t="inlineStr"/>
       <c r="Q177" s="8" t="inlineStr">
         <is>
-          <t>olympus_insights, PulseAction, alerts</t>
+          <t>Sent notifications</t>
         </is>
       </c>
       <c r="R177" s="8" t="inlineStr">
         <is>
-          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
+          <t>notification_queue table</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -31053,12 +31312,12 @@
     <row r="178" ht="30" customHeight="1">
       <c r="A178" s="8" t="inlineStr">
         <is>
-          <t>practice_status_listener</t>
-        </is>
-      </c>
-      <c r="B178" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>olympus_heartbeat</t>
+        </is>
+      </c>
+      <c r="B178" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C178" s="8" t="inlineStr">
@@ -31073,12 +31332,12 @@
       </c>
       <c r="E178" s="8" t="inlineStr">
         <is>
-          <t>continuo (event-driven)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F178" s="8" t="inlineStr">
         <is>
-          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
+          <t>Olympus DB Guardian heartbeat: lightweight PG health check, connection pool stats, replication lag detection.</t>
         </is>
       </c>
       <c r="G178" s="8" t="inlineStr">
@@ -31121,12 +31380,12 @@
       <c r="P178" s="8" t="inlineStr"/>
       <c r="Q178" s="8" t="inlineStr">
         <is>
-          <t>Practice state change events</t>
+          <t>Health metrics, PG stats</t>
         </is>
       </c>
       <c r="R178" s="8" t="inlineStr">
         <is>
-          <t>Redis pub/sub practice_status channel</t>
+          <t>PostgreSQL pg_stat_statements</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -31134,12 +31393,12 @@
     <row r="179" ht="30" customHeight="1">
       <c r="A179" s="8" t="inlineStr">
         <is>
-          <t>proactive_compliance_monitor</t>
-        </is>
-      </c>
-      <c r="B179" s="9" t="inlineStr">
-        <is>
-          <t>CRM</t>
+          <t>olympus_pulse</t>
+        </is>
+      </c>
+      <c r="B179" s="18" t="inlineStr">
+        <is>
+          <t>Olympus</t>
         </is>
       </c>
       <c r="C179" s="8" t="inlineStr">
@@ -31154,12 +31413,12 @@
       </c>
       <c r="E179" s="8" t="inlineStr">
         <is>
-          <t>ogni 24h (86400s)</t>
+          <t>ogni 6h</t>
         </is>
       </c>
       <c r="F179" s="8" t="inlineStr">
         <is>
-          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
+          <t>Olympus DB Guardian full pulse: vacuum analysis, bloat intelligence, query regression detection (&gt;30%), autovacuum advisor, partition-aware cleanup.</t>
         </is>
       </c>
       <c r="G179" s="8" t="inlineStr">
@@ -31202,12 +31461,12 @@
       <c r="P179" s="8" t="inlineStr"/>
       <c r="Q179" s="8" t="inlineStr">
         <is>
-          <t>Compliance alerts (WhatsApp/Telegram)</t>
+          <t>olympus_insights, PulseAction, alerts</t>
         </is>
       </c>
       <c r="R179" s="8" t="inlineStr">
         <is>
-          <t>CRM practices, client documents</t>
+          <t>pg_stat_statements, pg_stat_user_tables, index stats</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -31215,7 +31474,7 @@
     <row r="180" ht="30" customHeight="1">
       <c r="A180" s="8" t="inlineStr">
         <is>
-          <t>team_timesheet_auto_logout</t>
+          <t>practice_status_listener</t>
         </is>
       </c>
       <c r="B180" s="9" t="inlineStr">
@@ -31235,12 +31494,12 @@
       </c>
       <c r="E180" s="8" t="inlineStr">
         <is>
-          <t>ogni 5min (300s)</t>
+          <t>continuo (event-driven)</t>
         </is>
       </c>
       <c r="F180" s="8" t="inlineStr">
         <is>
-          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
+          <t>Practice status listener: listens for CRM practice state changes via Redis pub/sub, triggers follow-up actions (reminders, escalations).</t>
         </is>
       </c>
       <c r="G180" s="8" t="inlineStr">
@@ -31283,12 +31542,12 @@
       <c r="P180" s="8" t="inlineStr"/>
       <c r="Q180" s="8" t="inlineStr">
         <is>
-          <t>Auto-closed timesheet sessions</t>
+          <t>Practice state change events</t>
         </is>
       </c>
       <c r="R180" s="8" t="inlineStr">
         <is>
-          <t>work_sessions table</t>
+          <t>Redis pub/sub practice_status channel</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -31296,7 +31555,7 @@
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="8" t="inlineStr">
         <is>
-          <t>weekly_email_reporter</t>
+          <t>proactive_compliance_monitor</t>
         </is>
       </c>
       <c r="B181" s="9" t="inlineStr">
@@ -31316,12 +31575,12 @@
       </c>
       <c r="E181" s="8" t="inlineStr">
         <is>
-          <t>Dom 16:00 WITA</t>
+          <t>ogni 24h (86400s)</t>
         </is>
       </c>
       <c r="F181" s="8" t="inlineStr">
         <is>
-          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
+          <t>Proactive compliance: daily scan of all clients for document expiry, visa deadlines, LKPM due dates. Sends automated WhatsApp/Telegram alerts.</t>
         </is>
       </c>
       <c r="G181" s="8" t="inlineStr">
@@ -31364,25 +31623,29 @@
       <c r="P181" s="8" t="inlineStr"/>
       <c r="Q181" s="8" t="inlineStr">
         <is>
-          <t>Weekly team email report</t>
+          <t>Compliance alerts (WhatsApp/Telegram)</t>
         </is>
       </c>
       <c r="R181" s="8" t="inlineStr">
         <is>
-          <t>email_logs, team_members tables</t>
-        </is>
-      </c>
-      <c r="S181" s="8" t="inlineStr"/>
+          <t>CRM practices, client documents</t>
+        </is>
+      </c>
+      <c r="S181" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — _init_background_services() commented out. Re-enable when omnichannel stabilization complete.</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="30" customHeight="1">
       <c r="A182" s="8" t="inlineStr">
         <is>
-          <t>workflow_queue</t>
-        </is>
-      </c>
-      <c r="B182" s="11" t="inlineStr">
-        <is>
-          <t>Ops</t>
+          <t>team_timesheet_auto_logout</t>
+        </is>
+      </c>
+      <c r="B182" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C182" s="8" t="inlineStr">
@@ -31397,12 +31660,12 @@
       </c>
       <c r="E182" s="8" t="inlineStr">
         <is>
-          <t>continuo (poll su tabella jobs)</t>
+          <t>ogni 5min (300s)</t>
         </is>
       </c>
       <c r="F182" s="8" t="inlineStr">
         <is>
-          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+          <t>Team timesheet auto-logout: checks for expired work sessions every 5min, auto-closes sessions that exceeded 10h without checkout.</t>
         </is>
       </c>
       <c r="G182" s="8" t="inlineStr">
@@ -31445,12 +31708,12 @@
       <c r="P182" s="8" t="inlineStr"/>
       <c r="Q182" s="8" t="inlineStr">
         <is>
-          <t>Completed workflow results</t>
+          <t>Auto-closed timesheet sessions</t>
         </is>
       </c>
       <c r="R182" s="8" t="inlineStr">
         <is>
-          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+          <t>work_sessions table</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -31458,12 +31721,12 @@
     <row r="183" ht="30" customHeight="1">
       <c r="A183" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_digest_loop</t>
-        </is>
-      </c>
-      <c r="B183" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>websocket_redis_listener</t>
+        </is>
+      </c>
+      <c r="B183" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
         </is>
       </c>
       <c r="C183" s="8" t="inlineStr">
@@ -31478,12 +31741,12 @@
       </c>
       <c r="E183" s="8" t="inlineStr">
         <is>
-          <t>ogni N ore (configurable)</t>
+          <t>continuo (Redis→WebSocket bridge)</t>
         </is>
       </c>
       <c r="F183" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+          <t>WebSocket Redis bridge: persistent background task that relays Redis pub/sub messages to connected WebSocket clients for real-time UI updates.</t>
         </is>
       </c>
       <c r="G183" s="8" t="inlineStr">
@@ -31526,12 +31789,12 @@
       <c r="P183" s="8" t="inlineStr"/>
       <c r="Q183" s="8" t="inlineStr">
         <is>
-          <t>Twitter digest report</t>
+          <t>Real-time WebSocket messages to frontend</t>
         </is>
       </c>
       <c r="R183" s="8" t="inlineStr">
         <is>
-          <t>Stored Twitter matches</t>
+          <t>Redis pub/sub channels</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -31539,12 +31802,12 @@
     <row r="184" ht="30" customHeight="1">
       <c r="A184" s="8" t="inlineStr">
         <is>
-          <t>x_monitor_run_loop</t>
-        </is>
-      </c>
-      <c r="B184" s="19" t="inlineStr">
-        <is>
-          <t>Garuda</t>
+          <t>weekly_email_reporter</t>
+        </is>
+      </c>
+      <c r="B184" s="9" t="inlineStr">
+        <is>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C184" s="8" t="inlineStr">
@@ -31559,12 +31822,12 @@
       </c>
       <c r="E184" s="8" t="inlineStr">
         <is>
-          <t>ogni N minuti (configurable)</t>
+          <t>Dom 16:00 WITA</t>
         </is>
       </c>
       <c r="F184" s="8" t="inlineStr">
         <is>
-          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+          <t>Weekly email report: sends Sunday digest with individual team member email activity metrics.</t>
         </is>
       </c>
       <c r="G184" s="8" t="inlineStr">
@@ -31607,17 +31870,264 @@
       <c r="P184" s="8" t="inlineStr"/>
       <c r="Q184" s="8" t="inlineStr">
         <is>
+          <t>Weekly team email report</t>
+        </is>
+      </c>
+      <c r="R184" s="8" t="inlineStr">
+        <is>
+          <t>email_logs, team_members tables</t>
+        </is>
+      </c>
+      <c r="S184" s="8" t="inlineStr"/>
+    </row>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="8" t="inlineStr">
+        <is>
+          <t>workflow_queue</t>
+        </is>
+      </c>
+      <c r="B185" s="11" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="C185" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E185" s="8" t="inlineStr">
+        <is>
+          <t>continuo (poll su tabella jobs)</t>
+        </is>
+      </c>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>Workflow job queue: PG SKIP LOCKED + LangGraph checkpointer. Processes async workflows (document generation, complex multi-step operations).</t>
+        </is>
+      </c>
+      <c r="G185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I185" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L185" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M185" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N185" s="8" t="inlineStr"/>
+      <c r="O185" s="8" t="inlineStr"/>
+      <c r="P185" s="8" t="inlineStr"/>
+      <c r="Q185" s="8" t="inlineStr">
+        <is>
+          <t>Completed workflow results</t>
+        </is>
+      </c>
+      <c r="R185" s="8" t="inlineStr">
+        <is>
+          <t>workflow_jobs table (PG SKIP LOCKED)</t>
+        </is>
+      </c>
+      <c r="S185" s="8" t="inlineStr"/>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_digest_loop</t>
+        </is>
+      </c>
+      <c r="B186" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C186" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D186" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E186" s="8" t="inlineStr">
+        <is>
+          <t>ogni N ore (configurable)</t>
+        </is>
+      </c>
+      <c r="F186" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter digest: periodic summary of matched tweets, sends digest report.</t>
+        </is>
+      </c>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I186" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L186" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M186" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N186" s="8" t="inlineStr"/>
+      <c r="O186" s="8" t="inlineStr"/>
+      <c r="P186" s="8" t="inlineStr"/>
+      <c r="Q186" s="8" t="inlineStr">
+        <is>
+          <t>Twitter digest report</t>
+        </is>
+      </c>
+      <c r="R186" s="8" t="inlineStr">
+        <is>
+          <t>Stored Twitter matches</t>
+        </is>
+      </c>
+      <c r="S186" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — same as x_monitor_run_loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="8" t="inlineStr">
+        <is>
+          <t>x_monitor_run_loop</t>
+        </is>
+      </c>
+      <c r="B187" s="19" t="inlineStr">
+        <is>
+          <t>Garuda</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t>Fly.io</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="inlineStr">
+        <is>
+          <t>backend-loop</t>
+        </is>
+      </c>
+      <c r="E187" s="8" t="inlineStr">
+        <is>
+          <t>ogni N minuti (configurable)</t>
+        </is>
+      </c>
+      <c r="F187" s="8" t="inlineStr">
+        <is>
+          <t>X/Twitter monitor: polls Twitter API for keyword matches (Bali business, visa, immigration), stores matches for analysis.</t>
+        </is>
+      </c>
+      <c r="G187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I187" s="8" t="inlineStr">
+        <is>
+          <t>Health Monitor</t>
+        </is>
+      </c>
+      <c r="J187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L187" s="15" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="M187" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N187" s="8" t="inlineStr"/>
+      <c r="O187" s="8" t="inlineStr"/>
+      <c r="P187" s="8" t="inlineStr"/>
+      <c r="Q187" s="8" t="inlineStr">
+        <is>
           <t>Twitter match entries</t>
         </is>
       </c>
-      <c r="R184" s="8" t="inlineStr">
+      <c r="R187" s="8" t="inlineStr">
         <is>
           <t>Twitter API v2 search/recent</t>
         </is>
       </c>
-      <c r="S184" s="8" t="inlineStr">
-        <is>
-          <t>CRC broken — X API access issues</t>
+      <c r="S187" s="8" t="inlineStr">
+        <is>
+          <t>DISABLED — loops exist in code but no startup wiring in service_initializer.py. X/Twitter CRC also broken.</t>
         </is>
       </c>
     </row>

</xml_diff>